<commit_message>
bug fixes post migration to DuckDB
</commit_message>
<xml_diff>
--- a/.cursor/docs/FullAppDocumentation.xlsx
+++ b/.cursor/docs/FullAppDocumentation.xlsx
@@ -696,12 +696,12 @@
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>Raw .xlsx, .csv, .xlsm, .xltx files or a .zip containing them.</t>
+          <t>ZIP archive, folder, or individual CSV / Excel files (.xlsx, .xlsm, .xlsb, .xltx, .xltm). ZIP files inside folders are automatically extracted (one level deep).</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>Files parsed with python-calamine for Excel (header=None), CSV with header=None. Each sheet becomes a separate table (filename::sheetname). Raw data stored in raw__* and processed data in tbl__* tables in a session SQLite DB. Inventory and previews are built.</t>
+          <t>ZIP extracted, each Excel/CSV read into a pandas DataFrame. Raw table created via DuckDB native DataFrame register (zero-copy, no Python row iteration). Data table built from raw table via SQL CREATE TABLE AS SELECT with ROW_NUMBER() to skip header row and filter empty rows. Tables registered in session registry. Single COMMIT at end.</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
@@ -795,7 +795,7 @@
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Fetches up to 1000 rows from SQLite (SELECT * LIMIT 1000), then pick_best_rows() scores each row by counting non-null non-empty columns and returns the top 50 most populated rows. This ensures previews show the most informative data rather than whatever happened to be first.</t>
+          <t>Inventory, files payload, and previews built using batched SQL queries against information_schema (column lists and row counts fetched for all tables in two queries instead of per-table loops). Distinct values per column fetched via a single UNION ALL query across all columns.</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
@@ -2029,7 +2029,7 @@
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>Per-file date format detection (dominant format, format percentages, examples, consistency flag). If spend and date columns available: year × month spend pivot table. AI generates insight bullets.</t>
+          <t>All CAST(SUBSTR(...) AS INTEGER) replaced with TRY_CAST for safe conversion of potentially non-date strings. The strftime fallback also wraps its input in TRY_CAST(... AS TIMESTAMP). Table resolution falls back to final_merged if the versioned table (final_merged_vX) is not found.</t>
         </is>
       </c>
       <c r="F30" s="4" t="inlineStr">
@@ -2051,7 +2051,7 @@
       </c>
       <c r="I30" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>TRY_CAST instead of CAST for date extraction</t>
         </is>
       </c>
     </row>
@@ -2438,12 +2438,12 @@
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>Files are parsed (CSV with UTF-8 BOM strip, Excel via openpyxl). Headers are uppercased and deduped. A session SQLite DB is created. Raw data is stored in raw__* tables and typed data in data__* tables. Column info (names + up to 50 sample values) is collected.</t>
+          <t>ZIP or single file parsed. Each Excel sheet/CSV read into a pandas DataFrame (not a Python grid). Raw table created via DuckDB native DataFrame register (zero-copy). Data table built from raw table via SQL CREATE TABLE AS SELECT with ROW_NUMBER() to skip header row and filter empty rows. Session connections are now cached in an LRU OrderedDict. Tables registered in session. Single COMMIT at end.</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
-          <t>sessionId, columns, fileInventory, previews, warnings (for files that failed to parse).</t>
+          <t>Session ID, table keys list, warnings list</t>
         </is>
       </c>
       <c r="G2" s="4" t="inlineStr">
@@ -2564,7 +2564,7 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>Fetches up to 1000 rows from SQLite (SELECT * LIMIT 1000), then pick_best_rows() scores each row by counting non-null non-empty columns and returns the top 50 most populated rows. This ensures previews show the most informative data.</t>
+          <t>Inventory built via batched SQL queries: column counts and row counts fetched for all tables in two queries (information_schema GROUP BY + UNION ALL of COUNTs) instead of per-table loops. Column info gathered with batched information_schema query.</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr">
@@ -2606,7 +2606,7 @@
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>raw__* table is re-read, the chosen row becomes the header, data__* table is rebuilt, column info and inventory are refreshed.</t>
+          <t>Only the chosen header row is fetched from the raw table via SQL with ROW_NUMBER(). Data table is rebuilt entirely in SQL (CREATE TABLE AS SELECT) skipping the header row and empty rows. No Python iteration over the full table.</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
@@ -2732,8 +2732,7 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>Pass 1 (Deterministic): Case-insensitive exact match of column names against 31 standard procurement field names and their aliases.
-Pass 2 (AI): For each unmatched standard field, a parallel AI call (up to 8 concurrent) sends all remaining unmatched columns with samples to the LLM.</t>
+          <t>Deterministic matching first (exact name + fuzzy token-based matching with type compatibility checks), then parallel per-field AI calls for remaining fields. AI receives enriched column statistics (inferred type, null rate, distinct count, total rows) and a comprehensive system prompt listing all 31 standard fields. Post-AI validation resolves conflicts where two fields claim the same column, checks column existence, and verifies type compatibility.</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
@@ -2819,7 +2818,7 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>All data__* tables are concatenated into one DataFrame. Types are cast (numeric cleaning, date parsing with DMY/MDY profiling and Excel serial handling, strings stripped). Result is written to analysis_data table. Rows missing total_spend or invoice_date go to _null_rows. A castReport is generated showing parse % and null counts per field.</t>
+          <t>Saves mapping, builds analysis_data table with enforced types. DuckDB DataFrame registration is wrapped in try/finally to prevent resource leaks if table creation fails. Critical null audit creates _null_rows table for rows missing total_spend or invoice_date.</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
@@ -2861,9 +2860,7 @@
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>(A) Date Pivot: SQL aggregation of total_spend by year/month from invoice_date.
-(B) Pareto Analysis: Rows sorted by spend descending; cumulative thresholds at 80/85/90/95/99% tracking supplier count, transaction count, and unique vendor+description pairs.
-(C) Description Quality: For each mapped description column (invoice, PO, material, GL), SQL stats are computed (avg length, multi-word count/spend, null-proxy count/spend, total populated/spend). Up to 4 AI calls are made — one per description column that has data.</t>
+          <t>Date-spend pivot uses TRY_CAST for safe VARCHAR-to-TIMESTAMP conversion. Pareto analysis uses SQL window functions (SUM OVER ORDER BY) for cumulative calculations instead of fetching all rows to Python. Zero-division guards and type coercion applied throughout. Metrics extraction failures are logged rather than silently swallowed.</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
@@ -2993,7 +2990,7 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>Frontend renders from stored view_results — no new backend call needed.</t>
+          <t>View engine loads analysis_data and explicitly coerces known string columns (supplier_name, currency_code, etc.) to str and numeric columns (total_spend) to pd.to_numeric. All percentage-of-total calculations use max(total, 1e-9) to prevent division by zero. Datetime column detection uses pd.api.types.is_datetime64_any_dtype for robustness.</t>
         </is>
       </c>
       <c r="F15" s="5" t="inlineStr">
@@ -3449,7 +3446,7 @@
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>Receives file via POST. Extracts session ID from form data. Opens per-session SQLite database via get_session_db(). Clears any prior tables. Parses ZIP/Excel/CSV using pandas (temporary DataFrames). For each sheet/file, writes raw and data copies to SQLite via df_to_sqlite(), registers in table_registry. Frees DataFrames after writing. Returns inventory list.</t>
+          <t>ZIP or single file parsed. Each Excel sheet/CSV read into a pandas DataFrame. Raw table written once using DuckDB native DataFrame register (zero-copy). Data table created from raw via SQL CREATE TABLE AS SELECT (no second Python write). Tables registered in session. Single COMMIT at end.</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
@@ -3637,7 +3634,7 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>Fetches up to 1000 rows from SQLite via sqlite_to_df(limit=1000), then pick_best_df_rows() scores each row by counting non-null non-empty columns and returns the top 50 most populated rows. This ensures previews show the most informative data.</t>
+          <t>Inventory built via batched SQL queries: column counts and row counts fetched for all tables in two queries (information_schema GROUP BY + UNION ALL of COUNTs) instead of per-table loops.</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
@@ -3731,7 +3728,7 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>Loads data table from SQLite via sqlite_to_df(). Drops rows by index. Saves modified DataFrame back to SQLite via df_to_sqlite().</t>
+          <t>Rebuilds the table in pure SQL using ROW_NUMBER() to exclude the selected row indices, then renames the result back. No pandas round-trip.</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
@@ -3825,7 +3822,7 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>Loads full data table from SQLite via sqlite_to_df(). Copies it to the "active" table via df_to_sqlite(conn, "active", df). Stores active_table_key and filename in meta table. Triggers background XLSX cache generation to disk.</t>
+          <t>Copies the selected data table to the active table using a pure SQL CREATE TABLE AS SELECT (no pandas round-trip). Stores the table key and filename in session metadata. Returns a row count and a small preview.</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
@@ -3872,7 +3869,7 @@
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>Loads the active table from SQLite via sqlite_to_df(conn, "active"). Runs _suggest_columns() heuristic on the DataFrame to score date, currency, and spend columns by header keywords and value patterns.</t>
+          <t>Reads a 200-row sample from the active table (not the full table) and uses header keywords plus content heuristics to suggest the best date, currency, and spend columns.</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
@@ -4384,7 +4381,7 @@
       </c>
       <c r="B22" s="9" t="inlineStr">
         <is>
-          <t>Download Excel</t>
+          <t>Download CSV</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
@@ -4399,17 +4396,17 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>Reads session ID from query params. Checks for a pre-built XLSX cache file on disk (generated in background after each normalization). If found, serves from disk. If not found or still building, loads the active table from SQLite via sqlite_to_df() and builds XLSX on the fly using openpyxl write_only mode.</t>
+          <t>Reads the active table from DuckDB, converts it to CSV in memory, and streams it as a file download. No background caching or pre-generation.</t>
         </is>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>XLSX file stream ({basename}_normalized.xlsx).</t>
+          <t>CSV file bytes</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>Browser downloads an .xlsx file of the full normalized dataset.</t>
+          <t>Browser downloads a .csv file named {filename}_normalized.csv</t>
         </is>
       </c>
       <c r="H22" s="5" t="inlineStr">

</xml_diff>

<commit_message>
updated data quality analysis in mod 3
</commit_message>
<xml_diff>
--- a/.cursor/docs/FullAppDocumentation.xlsx
+++ b/.cursor/docs/FullAppDocumentation.xlsx
@@ -617,7 +617,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I39"/>
+  <dimension ref="A1:I43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1008,98 +1008,98 @@
       </c>
     </row>
     <row r="9" ht="100" customHeight="1">
-      <c r="A9" s="8" t="inlineStr">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2. Data Preview</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Bulk delete tables</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Select tables via checkboxes (individual or Select All), then click Delete Selected and confirm.</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Set of table_key strings for tables to delete</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Calls the existing /delete-table endpoint for each selected table in sequence. Each call drops the DuckDB tables and removes the registry entry.</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Updated inventory and previews after each deletion</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Selected tables disappear from the list. The bulk selection bar and checkboxes reset.</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="100" customHeight="1">
+      <c r="A10" s="8" t="inlineStr">
         <is>
           <t>3. Append Strategy</t>
         </is>
       </c>
-      <c r="B9" s="9" t="inlineStr">
+      <c r="B10" s="9" t="inlineStr">
         <is>
           <t>Generate Append Plan</t>
         </is>
       </c>
-      <c r="C9" s="5" t="inlineStr">
+      <c r="C10" s="5" t="inlineStr">
         <is>
           <t>User clicks "Generate Append Plan".</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
+      <c r="D10" s="5" t="inlineStr">
         <is>
           <t>sessionId, apiKey. Backend reads filesPayload (column names, row counts, up to 10 distinct examples per column, column overlap scores between all table pairs).</t>
         </is>
       </c>
-      <c r="E9" s="5" t="inlineStr">
+      <c r="E10" s="5" t="inlineStr">
         <is>
           <t>Batches of up to 25 tables per AI call. AI analyzes column overlap, value overlap, file types, and column headers to group tables that should be stacked (appended). Tables with 100% or near-100% column match are grouped. Low-overlap tables go to unassigned. Each group gets a descriptive name and reason.</t>
         </is>
       </c>
-      <c r="F9" s="5" t="inlineStr">
+      <c r="F10" s="5" t="inlineStr">
         <is>
           <t>appendGroups (list of groups with group_id, group_name, tables, reason), unassigned (list with table_key, reason), notes.</t>
         </is>
       </c>
-      <c r="G9" s="5" t="inlineStr">
+      <c r="G10" s="5" t="inlineStr">
         <is>
           <t>Group cards showing file names, AI-generated group name and reason. Unassigned files shown as chips. User can rename groups, move files between groups, exclude files.</t>
         </is>
       </c>
-      <c r="H9" s="5" t="inlineStr">
+      <c r="H10" s="5" t="inlineStr">
         <is>
           <t>System: "You analyze extracted tables and decide which should be APPENDED (union/stacked)..." (full prompt covers column overlap rules, value overlap, file type handling, empty table handling, group naming).
 User: JSON payload of all tables with columns, distinct examples, overlap scores.
 Response: {append_groups, unassigned, notes}.</t>
         </is>
       </c>
-      <c r="I9" s="5" t="inlineStr">
+      <c r="I10" s="5" t="inlineStr">
         <is>
           <t>MAX_TABLES_PER_CALL = 25. EXAMPLES_PER_COLUMN = 10. MAX_COLUMNS_IN_FILES_PAYLOAD = 300. MAX_COLUMNS_FOR_DISTINCT_EXAMPLES = 40. MAX_DISTINCT_VALUES_PER_COLUMN = 50.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="100" customHeight="1">
-      <c r="A10" s="8" t="inlineStr">
-        <is>
-          <t>3. Append Strategy</t>
-        </is>
-      </c>
-      <c r="B10" s="9" t="inlineStr">
-        <is>
-          <t>Edit groups manually</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>User renames groups, moves tables between groups, creates new groups from selected tables, excludes tables.</t>
-        </is>
-      </c>
-      <c r="D10" s="4" t="inlineStr">
-        <is>
-          <t>Updated appendGroups and unassigned arrays.</t>
-        </is>
-      </c>
-      <c r="E10" s="4" t="inlineStr">
-        <is>
-          <t>POST /api/save-append-groups persists the updated groups. Group names are synced to schema meta.</t>
-        </is>
-      </c>
-      <c r="F10" s="4" t="inlineStr">
-        <is>
-          <t>Confirmation.</t>
-        </is>
-      </c>
-      <c r="G10" s="4" t="inlineStr">
-        <is>
-          <t>Groups update in real-time. Fire-and-forget save.</t>
-        </is>
-      </c>
-      <c r="H10" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="I10" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
         </is>
       </c>
     </row>
@@ -1111,131 +1111,178 @@
       </c>
       <c r="B11" s="9" t="inlineStr">
         <is>
+          <t>Edit groups manually</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>User renames groups, moves tables between groups, creates new groups from selected tables, excludes tables.</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>Updated appendGroups and unassigned arrays.</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>POST /api/save-append-groups persists the updated groups. Group names are synced to schema meta.</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>Confirmation.</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>Groups update in real-time. Fire-and-forget save.</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I11" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="100" customHeight="1">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>3. Append Strategy</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
           <t>Analyze Header Alignment (Mapping)</t>
         </is>
       </c>
-      <c r="C11" s="5" t="inlineStr">
+      <c r="C12" s="5" t="inlineStr">
         <is>
           <t>User clicks "Analyze Header Alignment".</t>
         </is>
       </c>
-      <c r="D11" s="5" t="inlineStr">
+      <c r="D12" s="5" t="inlineStr">
         <is>
           <t>appendGroups with table details.</t>
         </is>
       </c>
-      <c r="E11" s="5" t="inlineStr">
+      <c r="E12" s="5" t="inlineStr">
         <is>
           <t>Per group with ≥2 non-empty tables: AI produces a canonical schema and per-table column mapping (which source column maps to which canonical column). Single-table groups get identity mapping.</t>
         </is>
       </c>
-      <c r="F11" s="5" t="inlineStr">
+      <c r="F12" s="5" t="inlineStr">
         <is>
           <t>appendGroupMappings per group: canonical_schema, per_table (column_mapping, missing_canonical, extra_source, confidence, notes).</t>
         </is>
       </c>
-      <c r="G11" s="5" t="inlineStr">
+      <c r="G12" s="5" t="inlineStr">
         <is>
           <t>Mapping table per group showing canonical columns and how each source table's columns align. User can edit mappings via dropdowns.</t>
         </is>
       </c>
-      <c r="H11" s="5" t="inlineStr">
+      <c r="H12" s="5" t="inlineStr">
         <is>
           <t>System: "You are a schema alignment engine for APPENDING (union/stacking)..." (covers exact match, fuzzy match, value similarity rules).
 User: Group details with columns and distinct examples.
 Response: {group_id, canonical_schema, per_table, notes}.</t>
         </is>
       </c>
-      <c r="I11" s="5" t="inlineStr">
+      <c r="I12" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="100" customHeight="1">
-      <c r="A12" s="8" t="inlineStr">
+    <row r="13" ht="100" customHeight="1">
+      <c r="A13" s="8" t="inlineStr">
         <is>
           <t>3. Append Strategy</t>
         </is>
       </c>
-      <c r="B12" s="9" t="inlineStr">
+      <c r="B13" s="9" t="inlineStr">
         <is>
           <t>Execute Append &amp; Stack</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="C13" s="4" t="inlineStr">
         <is>
           <t>User clicks "Execute Append &amp; Stack".</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr">
+      <c r="D13" s="4" t="inlineStr">
         <is>
           <t>appendGroupMappings, unassignedTables.</t>
         </is>
       </c>
-      <c r="E12" s="4" t="inlineStr">
+      <c r="E13" s="4" t="inlineStr">
         <is>
           <t>Per group: CREATE TABLE appended__{group_id} with all canonical columns (TEXT type) + _source_table column. INSERT...SELECT from each source table with NULLs for missing canonical columns. Unassigned tables copied as appended__{table_key}. groupSchemaTableRows meta updated.</t>
         </is>
       </c>
-      <c r="F12" s="4" t="inlineStr">
+      <c r="F13" s="4" t="inlineStr">
         <is>
           <t>appendReport (per-group row counts, column counts), groupSchema.</t>
         </is>
       </c>
-      <c r="G12" s="4" t="inlineStr">
+      <c r="G13" s="4" t="inlineStr">
         <is>
           <t>Append report card showing per-group results (rows, columns, sources). "Proceed to Header Normalisation" button.</t>
         </is>
       </c>
-      <c r="H12" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="I12" s="4" t="inlineStr">
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I13" s="4" t="inlineStr">
         <is>
           <t>All columns stored as TEXT.</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="100" customHeight="1">
-      <c r="A13" s="10" t="inlineStr">
+    <row r="14" ht="100" customHeight="1">
+      <c r="A14" s="10" t="inlineStr">
         <is>
           <t>4. Header Norm</t>
         </is>
       </c>
-      <c r="B13" s="11" t="inlineStr">
+      <c r="B14" s="11" t="inlineStr">
         <is>
           <t>Run Header Normalisation</t>
         </is>
       </c>
-      <c r="C13" s="5" t="inlineStr">
+      <c r="C14" s="5" t="inlineStr">
         <is>
           <t>User clicks "Run Header Normalisation" (requires API key).</t>
         </is>
       </c>
-      <c r="D13" s="5" t="inlineStr">
+      <c r="D14" s="5" t="inlineStr">
         <is>
           <t>sessionId, apiKey. Backend reads appended tables (or tbl__* if no append).</t>
         </is>
       </c>
-      <c r="E13" s="5" t="inlineStr">
+      <c r="E14" s="5" t="inlineStr">
         <is>
           <t>8-tier matching engine: (1) exact name match, (2) alias match from knowledge base, (3) fuzzy match (threshold 62), (4) semantic tag match, (5) type + pattern match, (6) description match, (7) learned alias match, (8) AI mapping. AI runs on unmatched columns with column name, samples, data type, null %, distinct %, neighbouring columns, and top-5 deterministic hints. Optional AI validation on mapped columns.</t>
         </is>
       </c>
-      <c r="F13" s="5" t="inlineStr">
+      <c r="F14" s="5" t="inlineStr">
         <is>
           <t>headerNormDecisions per group: each column gets an action (AUTO/KEEP/DROP), a mapped standard field name (or null), confidence, source tier, alternatives.</t>
         </is>
       </c>
-      <c r="G13" s="5" t="inlineStr">
+      <c r="G14" s="5" t="inlineStr">
         <is>
           <t>Per-group table with columns: action (AUTO/KEEP/DROP toggle), source column, mapped standard field (dropdown), confidence score, sample data rows. User can edit any decision.</t>
         </is>
       </c>
-      <c r="H13" s="5" t="inlineStr">
+      <c r="H14" s="5" t="inlineStr">
         <is>
           <t>Mapping — System: "You are a procurement data schema expert mapping source columns to a standard 73-field procurement taxonomy..." (covers field definitions, aliases, samples, deterministic hints, confidence guidelines).
 User: JSON with standard_fields, column metadata, deterministic_hints.
@@ -1244,56 +1291,9 @@
 Response: {idx, original_header, mapped_to, valid, confidence, reason}.</t>
         </is>
       </c>
-      <c r="I13" s="5" t="inlineStr">
+      <c r="I14" s="5" t="inlineStr">
         <is>
           <t>FUZZY_THRESHOLD = 62. AI_CONFIDENCE_THRESHOLD = 0.65. AI_VALIDATION_CONF_HIGH = 0.85. AI_VALIDATION_CONF_LOW = 0.65. AI map batch_size = 10. Validation batch = 20. max_workers = 2. Profile rows = 50.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="100" customHeight="1">
-      <c r="A14" s="10" t="inlineStr">
-        <is>
-          <t>4. Header Norm</t>
-        </is>
-      </c>
-      <c r="B14" s="11" t="inlineStr">
-        <is>
-          <t>Excel round-trip</t>
-        </is>
-      </c>
-      <c r="C14" s="4" t="inlineStr">
-        <is>
-          <t>User clicks "Download Excel" to get a template, edits decisions offline, then uploads the modified file.</t>
-        </is>
-      </c>
-      <c r="D14" s="4" t="inlineStr">
-        <is>
-          <t>Download: sessionId, groupId, decisions. Upload: Excel file.</t>
-        </is>
-      </c>
-      <c r="E14" s="4" t="inlineStr">
-        <is>
-          <t>Download builds an Excel with rows 1–3 as metadata (source column, current mapping, action) and 50 data rows. Upload parses decisions back from the workbook.</t>
-        </is>
-      </c>
-      <c r="F14" s="4" t="inlineStr">
-        <is>
-          <t>Download: Excel file. Upload: parsed decisions array.</t>
-        </is>
-      </c>
-      <c r="G14" s="4" t="inlineStr">
-        <is>
-          <t>Excel downloaded to browser. After upload, decisions table updates with the imported mappings.</t>
-        </is>
-      </c>
-      <c r="H14" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="I14" s="4" t="inlineStr">
-        <is>
-          <t>Excel template = 50 data rows.</t>
         </is>
       </c>
     </row>
@@ -1305,136 +1305,136 @@
       </c>
       <c r="B15" s="11" t="inlineStr">
         <is>
+          <t>Excel round-trip</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>User clicks "Download Excel" to get a template, edits decisions offline, then uploads the modified file.</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>Download: sessionId, groupId, decisions. Upload: Excel file.</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>Download builds an Excel with rows 1–3 as metadata (source column, current mapping, action) and 50 data rows. Upload parses decisions back from the workbook.</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>Download: Excel file. Upload: parsed decisions array.</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>Excel downloaded to browser. After upload, decisions table updates with the imported mappings.</t>
+        </is>
+      </c>
+      <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I15" s="4" t="inlineStr">
+        <is>
+          <t>Excel template = 50 data rows.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="100" customHeight="1">
+      <c r="A16" s="10" t="inlineStr">
+        <is>
+          <t>4. Header Norm</t>
+        </is>
+      </c>
+      <c r="B16" s="11" t="inlineStr">
+        <is>
           <t>Apply decisions</t>
         </is>
       </c>
-      <c r="C15" s="5" t="inlineStr">
+      <c r="C16" s="5" t="inlineStr">
         <is>
           <t>User clicks "Apply &amp; Proceed" (or "Skip to Data Cleaning").</t>
         </is>
       </c>
-      <c r="D15" s="5" t="inlineStr">
+      <c r="D16" s="5" t="inlineStr">
         <is>
           <t>decisions per group.</t>
         </is>
       </c>
-      <c r="E15" s="5" t="inlineStr">
+      <c r="E16" s="5" t="inlineStr">
         <is>
           <t>For each group, hn__* tables are created with renamed/mapped columns. Table registry updated to point to hn__* tables. Inventory and filesPayload refreshed.</t>
         </is>
       </c>
-      <c r="F15" s="5" t="inlineStr">
+      <c r="F16" s="5" t="inlineStr">
         <is>
           <t>Updated inventory, filesPayload with new column names.</t>
         </is>
       </c>
-      <c r="G15" s="5" t="inlineStr">
+      <c r="G16" s="5" t="inlineStr">
         <is>
           <t>User advances to Step 5. Table previews now show normalized column names.</t>
         </is>
       </c>
-      <c r="H15" s="5" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="I15" s="5" t="inlineStr">
+      <c r="H16" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I16" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="100" customHeight="1">
-      <c r="A16" s="12" t="inlineStr">
-        <is>
-          <t>5. Data Cleaning</t>
-        </is>
-      </c>
-      <c r="B16" s="13" t="inlineStr">
-        <is>
-          <t>5a — Basic Cleaning</t>
-        </is>
-      </c>
-      <c r="C16" s="4" t="inlineStr">
-        <is>
-          <t>User toggles options per group: remove null rows/cols, trim whitespace, case mode (upper/lower). Clicks "Apply Cleaning".</t>
-        </is>
-      </c>
-      <c r="D16" s="4" t="inlineStr">
-        <is>
-          <t>groupId, config (removeNullRows, removeNullColumns, caseMode, trimWhitespace).</t>
-        </is>
-      </c>
-      <c r="E16" s="4" t="inlineStr">
-        <is>
-          <t>In-place cleaning on the group's current SQL table: drop all-null rows, drop all-null columns, apply case transformation, trim whitespace.</t>
-        </is>
-      </c>
-      <c r="F16" s="4" t="inlineStr">
-        <is>
-          <t>Updated table with cleaning applied.</t>
-        </is>
-      </c>
-      <c r="G16" s="4" t="inlineStr">
-        <is>
-          <t>Preview refreshes showing cleaned data. Group marked as "done" in sidebar.</t>
-        </is>
-      </c>
-      <c r="H16" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="I16" s="4" t="inlineStr">
-        <is>
-          <t>Defaults: removeNullRows: true, removeNullColumns: true, caseMode: "upper", trimWhitespace: true.</t>
-        </is>
-      </c>
-    </row>
     <row r="17" ht="100" customHeight="1">
-      <c r="A17" s="12" t="inlineStr">
-        <is>
-          <t>5. Data Cleaning</t>
-        </is>
-      </c>
-      <c r="B17" s="13" t="inlineStr">
-        <is>
-          <t>5b — Deduplication</t>
-        </is>
-      </c>
-      <c r="C17" s="5" t="inlineStr">
-        <is>
-          <t>User selects key columns for dedup, clicks "Preview Stats" to see duplicate counts, then "Apply" to remove duplicates.</t>
-        </is>
-      </c>
-      <c r="D17" s="5" t="inlineStr">
-        <is>
-          <t>groupId, keyColumns.</t>
-        </is>
-      </c>
-      <c r="E17" s="5" t="inlineStr">
-        <is>
-          <t>Preview: counts exact duplicates on the selected composite key. Apply: removes duplicate rows keeping one per key.</t>
-        </is>
-      </c>
-      <c r="F17" s="5" t="inlineStr">
-        <is>
-          <t>Preview: duplicate counts and stats. Apply: updated row count.</t>
-        </is>
-      </c>
-      <c r="G17" s="5" t="inlineStr">
-        <is>
-          <t>Stats shown before apply (apply disabled until preview). After apply, preview refreshes.</t>
-        </is>
-      </c>
-      <c r="H17" s="5" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="I17" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>4. Header Norm</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Download mapping summary</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Click Download Mapping Summary in the toolbar.</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Current edited decisions (groupId to column decisions map) from frontend state</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>POST /header-norm-download-summary receives the decisions dict, builds an openpyxl Workbook with one sheet per group. Each sheet has two columns: Original Column Name and Mapped Column Name. Columns with action DROP are excluded. Returns the .xlsx as an attachment.</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Excel file (header_mapping_summary.xlsx) streamed as a download</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Browser downloads the Excel file automatically.</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>NA</t>
         </is>
       </c>
     </row>
@@ -1446,32 +1446,32 @@
       </c>
       <c r="B18" s="13" t="inlineStr">
         <is>
-          <t>5b — Column Standardization</t>
+          <t>5a — Basic Cleaning</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>User selects columns, clicks "Analyze" to detect leading zeros / numeric patterns, adjusts strip/pad/none per column, clicks "Apply".</t>
+          <t>User toggles options per group: remove null rows/cols, trim whitespace, case mode (upper/lower). Clicks "Apply Cleaning".</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>groupId, column names, action (strip/pad/none), pad length.</t>
+          <t>groupId, config (removeNullRows, removeNullColumns, caseMode, trimWhitespace).</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>Analyze: detects ≥90% numeric columns with ≥5% leading zeros. Apply: strips leading zeros or pads to specified length.</t>
+          <t>In-place cleaning on the group's current SQL table: drop all-null rows, drop all-null columns, apply case transformation, trim whitespace.</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>Analysis: per-column pattern stats. Apply: modified column values.</t>
+          <t>Updated table with cleaning applied.</t>
         </is>
       </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
-          <t>Analysis table showing pattern detection. User adjusts actions per column.</t>
+          <t>Preview refreshes showing cleaned data. Group marked as "done" in sidebar.</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
@@ -1481,7 +1481,7 @@
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>Leading zero detection: ≥90% numeric, ≥5% leading zeros. Pad length range: 1–50.</t>
+          <t>Defaults: removeNullRows: true, removeNullColumns: true, caseMode: "upper", trimWhitespace: true.</t>
         </is>
       </c>
     </row>
@@ -1493,32 +1493,32 @@
       </c>
       <c r="B19" s="13" t="inlineStr">
         <is>
-          <t>5b — Concatenation</t>
+          <t>5b — Deduplication</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>User picks 2+ columns in order, clicks "Apply" to create a new concatenated column.</t>
+          <t>User selects key columns for dedup, clicks "Preview Stats" to see duplicate counts, then "Apply" to remove duplicates.</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>groupId, ordered column list.</t>
+          <t>groupId, keyColumns.</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>New column created by concatenating selected columns with a separator.</t>
+          <t>Preview: counts exact duplicates on the selected composite key. Apply: removes duplicate rows keeping one per key.</t>
         </is>
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>New column added to table.</t>
+          <t>Preview: duplicate counts and stats. Apply: updated row count.</t>
         </is>
       </c>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>Preview shows the new column. User can delete concatenated columns.</t>
+          <t>Stats shown before apply (apply disabled until preview). After apply, preview refreshes.</t>
         </is>
       </c>
       <c r="H19" s="5" t="inlineStr">
@@ -1540,234 +1540,234 @@
       </c>
       <c r="B20" s="13" t="inlineStr">
         <is>
+          <t>5b — Column Standardization</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>User selects columns, clicks "Analyze" to detect leading zeros / numeric patterns, adjusts strip/pad/none per column, clicks "Apply".</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>groupId, column names, action (strip/pad/none), pad length.</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>Analyze: detects ≥90% numeric columns with ≥5% leading zeros. Apply: strips leading zeros or pads to specified length.</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>Analysis: per-column pattern stats. Apply: modified column values.</t>
+        </is>
+      </c>
+      <c r="G20" s="4" t="inlineStr">
+        <is>
+          <t>Analysis table showing pattern detection. User adjusts actions per column.</t>
+        </is>
+      </c>
+      <c r="H20" s="4" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I20" s="4" t="inlineStr">
+        <is>
+          <t>Leading zero detection: ≥90% numeric, ≥5% leading zeros. Pad length range: 1–50.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="100" customHeight="1">
+      <c r="A21" s="12" t="inlineStr">
+        <is>
+          <t>5. Data Cleaning</t>
+        </is>
+      </c>
+      <c r="B21" s="13" t="inlineStr">
+        <is>
+          <t>5b — Concatenation</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>User picks 2+ columns in order, clicks "Apply" to create a new concatenated column.</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>groupId, ordered column list.</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>New column created by concatenating selected columns with a separator.</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
+          <t>New column added to table.</t>
+        </is>
+      </c>
+      <c r="G21" s="5" t="inlineStr">
+        <is>
+          <t>Preview shows the new column. User can delete concatenated columns.</t>
+        </is>
+      </c>
+      <c r="H21" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I21" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="100" customHeight="1">
+      <c r="A22" s="12" t="inlineStr">
+        <is>
+          <t>5. Data Cleaning</t>
+        </is>
+      </c>
+      <c r="B22" s="13" t="inlineStr">
+        <is>
           <t>5b — Column Removal</t>
         </is>
       </c>
-      <c r="C20" s="4" t="inlineStr">
+      <c r="C22" s="4" t="inlineStr">
         <is>
           <t>User selects columns, clicks "Remove".</t>
         </is>
       </c>
-      <c r="D20" s="4" t="inlineStr">
+      <c r="D22" s="4" t="inlineStr">
         <is>
           <t>groupId, column names.</t>
         </is>
       </c>
-      <c r="E20" s="4" t="inlineStr">
+      <c r="E22" s="4" t="inlineStr">
         <is>
           <t>Columns removed from the SQL table with a backup for restore.</t>
         </is>
       </c>
-      <c r="F20" s="4" t="inlineStr">
+      <c r="F22" s="4" t="inlineStr">
         <is>
           <t>Columns removed. Restore option available.</t>
         </is>
       </c>
-      <c r="G20" s="4" t="inlineStr">
+      <c r="G22" s="4" t="inlineStr">
         <is>
           <t>Removed columns disappear from preview. "Restore" button per removed column.</t>
         </is>
       </c>
-      <c r="H20" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="I20" s="4" t="inlineStr">
+      <c r="H22" s="4" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I22" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="100" customHeight="1">
-      <c r="A21" s="14" t="inlineStr">
+    <row r="23" ht="100" customHeight="1">
+      <c r="A23" s="14" t="inlineStr">
         <is>
           <t>6. Merge</t>
         </is>
       </c>
-      <c r="B21" s="15" t="inlineStr">
+      <c r="B23" s="15" t="inlineStr">
         <is>
           <t>Recommend base table</t>
         </is>
       </c>
-      <c r="C21" s="5" t="inlineStr">
+      <c r="C23" s="5" t="inlineStr">
         <is>
           <t>Runs automatically on entering Step 6.</t>
         </is>
       </c>
-      <c r="D21" s="5" t="inlineStr">
+      <c r="D23" s="5" t="inlineStr">
         <is>
           <t>sessionId, apiKey.</t>
         </is>
       </c>
-      <c r="E21" s="5" t="inlineStr">
+      <c r="E23" s="5" t="inlineStr">
         <is>
           <t>Reads groupSchemaTableRows from session. If empty, returns prerequisite_missing: true with a message to complete Append Strategy first (no longer falsely reports session_expired). If one group, auto-selects. Otherwise uses AI to rank tables by row count, column count, and data quality.</t>
         </is>
       </c>
-      <c r="F21" s="5" t="inlineStr">
+      <c r="F23" s="5" t="inlineStr">
         <is>
           <t>recommended group ID, reasoning, rankings (all groups scored 0–100).</t>
         </is>
       </c>
-      <c r="G21" s="5" t="inlineStr">
+      <c r="G23" s="5" t="inlineStr">
         <is>
           <t>If prerequisite_missing, shows an Earlier Steps Required card with Back to Append Strategy button. Otherwise shows the AI recommendation with rankings.</t>
         </is>
       </c>
-      <c r="H21" s="5" t="inlineStr">
+      <c r="H23" s="5" t="inlineStr">
         <is>
           <t>System: "You are a data engineering assistant specialising in procurement data... decide which table is the best 'base' or 'fact' table for a LEFT JOIN merge workflow..." (covers cell count, row count, column richness, domain priority).
 User: Group metadata (row/col counts, column names, samples).
 Response: {recommended, reasoning, rankings}.</t>
         </is>
       </c>
-      <c r="I21" s="5" t="inlineStr">
+      <c r="I23" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="100" customHeight="1">
-      <c r="A22" s="14" t="inlineStr">
+    <row r="24" ht="100" customHeight="1">
+      <c r="A24" s="14" t="inlineStr">
         <is>
           <t>6. Merge</t>
         </is>
       </c>
-      <c r="B22" s="15" t="inlineStr">
+      <c r="B24" s="15" t="inlineStr">
         <is>
           <t>Common columns &amp; classification</t>
         </is>
       </c>
-      <c r="C22" s="4" t="inlineStr">
+      <c r="C24" s="4" t="inlineStr">
         <is>
           <t>Runs automatically when base and source are selected.</t>
         </is>
       </c>
-      <c r="D22" s="4" t="inlineStr">
+      <c r="D24" s="4" t="inlineStr">
         <is>
           <t>baseGroupId, sourceGroupId, apiKey, includePreview: true.</t>
         </is>
       </c>
-      <c r="E22" s="4" t="inlineStr">
+      <c r="E24" s="4" t="inlineStr">
         <is>
           <t>Normalized header matching → fuzzy match (cutoff 0.8) → value overlap on distinct sets (cap 2000 per column). Pairs kept if overlap &gt; 0.3; "strong" if ≥ 0.85. Unresolved columns classified by AI (identifier/descriptor/metric/weak) using 20 samples per column.</t>
         </is>
       </c>
-      <c r="F22" s="4" t="inlineStr">
+      <c r="F24" s="4" t="inlineStr">
         <is>
           <t>Per-column pair: match type, overlap score, classification (identifier/descriptor/metric/weak), eligibility (high/medium/low/never). Optional 50-row preview per group.</t>
         </is>
       </c>
-      <c r="G22" s="4" t="inlineStr">
+      <c r="G24" s="4" t="inlineStr">
         <is>
           <t>Side-by-side column tables for base and source. Matched columns highlighted. Classification badges. Key checkboxes for join key selection. Source columns clickable to "pull" (enrich).</t>
         </is>
       </c>
-      <c r="H22" s="4" t="inlineStr">
+      <c r="H24" s="4" t="inlineStr">
         <is>
           <t>Classification — System: "You are a procurement data expert... Classify this column into: identifier, descriptor, metric, weak..."
 User: Column name + 20 samples + COLUMN_METADATA reference.
 Response: {column_name, category, eligibility, reasoning, closest_standard_column}.</t>
         </is>
       </c>
-      <c r="I22" s="4" t="inlineStr">
+      <c r="I24" s="4" t="inlineStr">
         <is>
           <t>Fuzzy cutoff = 0.8. Distinct cap = 2000 per column. Overlap kept if &gt; 0.3. "Strong" if ≥ 0.85. Classification workers = 6. Sample values = 20 per column.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="100" customHeight="1">
-      <c r="A23" s="14" t="inlineStr">
-        <is>
-          <t>6. Merge</t>
-        </is>
-      </c>
-      <c r="B23" s="15" t="inlineStr">
-        <is>
-          <t>Select join keys</t>
-        </is>
-      </c>
-      <c r="C23" s="5" t="inlineStr">
-        <is>
-          <t>User checks key columns on both base and source sides (FIFO pairing: first base key pairs with first source key).</t>
-        </is>
-      </c>
-      <c r="D23" s="5" t="inlineStr">
-        <is>
-          <t>Selected base key columns, selected source key columns.</t>
-        </is>
-      </c>
-      <c r="E23" s="5" t="inlineStr">
-        <is>
-          <t>No backend call at this point — selection is frontend-only.</t>
-        </is>
-      </c>
-      <c r="F23" s="5" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="G23" s="5" t="inlineStr">
-        <is>
-          <t>Key selections shown with pairing summary. Composite key built from selected columns.</t>
-        </is>
-      </c>
-      <c r="H23" s="5" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="I23" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="100" customHeight="1">
-      <c r="A24" s="14" t="inlineStr">
-        <is>
-          <t>6. Merge</t>
-        </is>
-      </c>
-      <c r="B24" s="15" t="inlineStr">
-        <is>
-          <t>Select pull columns</t>
-        </is>
-      </c>
-      <c r="C24" s="4" t="inlineStr">
-        <is>
-          <t>User clicks source column headers to toggle "pull" (enrich from source).</t>
-        </is>
-      </c>
-      <c r="D24" s="4" t="inlineStr">
-        <is>
-          <t>Selected source columns to pull.</t>
-        </is>
-      </c>
-      <c r="E24" s="4" t="inlineStr">
-        <is>
-          <t>No backend call — frontend-only.</t>
-        </is>
-      </c>
-      <c r="F24" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="G24" s="4" t="inlineStr">
-        <is>
-          <t>Pulled columns highlighted on source side. Pull summary shown.</t>
-        </is>
-      </c>
-      <c r="H24" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="I24" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
         </is>
       </c>
     </row>
@@ -1779,32 +1779,32 @@
       </c>
       <c r="B25" s="15" t="inlineStr">
         <is>
-          <t>Simulate join</t>
+          <t>Select join keys</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>Runs automatically (debounced 500ms) after key/pull changes.</t>
+          <t>User checks key columns on both base and source sides (FIFO pairing: first base key pairs with first source key).</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>sessionId, baseGroupId, sourceGroupId, composite keys, pull columns.</t>
+          <t>Selected base key columns, selected source key columns.</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t>Creates slim temp tables with only key + pull columns. Builds composite key as TRIM(LOWER(CAST(col AS TEXT))) joined with '|||'. Computes match rate, explosion factor, unmatched counts on both sides, duplicate key counts on source.</t>
+          <t>No backend call at this point — selection is frontend-only.</t>
         </is>
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>matchRate, explosionFactor, unmatchedBase, unmatchedSource, duplicateSourceKeys.</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>Simulation stats card: match rate %, explosion factor, unmatched rows on each side. Warnings if low match or high explosion.</t>
+          <t>Key selections shown with pairing summary. Composite key built from selected columns.</t>
         </is>
       </c>
       <c r="H25" s="5" t="inlineStr">
@@ -1814,7 +1814,7 @@
       </c>
       <c r="I25" s="5" t="inlineStr">
         <is>
-          <t>Composite key separator = '|||'. Debounce = 500 ms.</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -1826,32 +1826,32 @@
       </c>
       <c r="B26" s="15" t="inlineStr">
         <is>
-          <t>Execute merge</t>
+          <t>Select pull columns</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>User clicks "Execute Merge".</t>
+          <t>User clicks source column headers to toggle "pull" (enrich from source).</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>sessionId, baseGroupId, sourceGroupId, keys, pulls, apiKey.</t>
+          <t>Selected source columns to pull.</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>Source dedup: on composite normalized key, keep MIN(rowid), drop blank keys. LEFT JOIN base to deduped source on composite key. Result written to _merge_step_{source_group_id}. Validation report generated. Result persisted as final_merged_v{n} and copied to final_merged. Merge history updated.</t>
+          <t>No backend call — frontend-only.</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>Streamed (SSE/NDJSON): progress events → final stats (rows, columns, match rate, new columns added) + merge_history entry.</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="G26" s="4" t="inlineStr">
         <is>
-          <t>Streaming progress card. On completion: "Merge Complete" hero with stats, column quality table, data preview. "What's Next" options: Redo, Another merge, Run DQA.</t>
+          <t>Pulled columns highlighted on source side. Pull summary shown.</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr">
@@ -1861,7 +1861,7 @@
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>MAX_ROW_MULTIPLIER = 1.02 (join ops). MIN_MATCH_RATE = 0.30 (warning threshold). CSV download chunk = fetchmany(2000).</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -1873,475 +1873,475 @@
       </c>
       <c r="B27" s="15" t="inlineStr">
         <is>
+          <t>Simulate join</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>Runs automatically (debounced 500ms) after key/pull changes.</t>
+        </is>
+      </c>
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>sessionId, baseGroupId, sourceGroupId, composite keys, pull columns.</t>
+        </is>
+      </c>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>Creates slim temp tables with only key + pull columns. Builds composite key as TRIM(LOWER(CAST(col AS TEXT))) joined with '|||'. Computes match rate, explosion factor, unmatched counts on both sides, duplicate key counts on source.</t>
+        </is>
+      </c>
+      <c r="F27" s="5" t="inlineStr">
+        <is>
+          <t>matchRate, explosionFactor, unmatchedBase, unmatchedSource, duplicateSourceKeys.</t>
+        </is>
+      </c>
+      <c r="G27" s="5" t="inlineStr">
+        <is>
+          <t>Simulation stats card: match rate %, explosion factor, unmatched rows on each side. Warnings if low match or high explosion.</t>
+        </is>
+      </c>
+      <c r="H27" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I27" s="5" t="inlineStr">
+        <is>
+          <t>Composite key separator = '|||'. Debounce = 500 ms.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="100" customHeight="1">
+      <c r="A28" s="14" t="inlineStr">
+        <is>
+          <t>6. Merge</t>
+        </is>
+      </c>
+      <c r="B28" s="15" t="inlineStr">
+        <is>
+          <t>Execute merge</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>User clicks "Execute Merge".</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>sessionId, baseGroupId, sourceGroupId, keys, pulls, apiKey.</t>
+        </is>
+      </c>
+      <c r="E28" s="4" t="inlineStr">
+        <is>
+          <t>Source dedup: on composite normalized key, keep MIN(rowid), drop blank keys. LEFT JOIN base to deduped source on composite key. Result written to _merge_step_{source_group_id}. Validation report generated. Result persisted as final_merged_v{n} and copied to final_merged. Merge history updated.</t>
+        </is>
+      </c>
+      <c r="F28" s="4" t="inlineStr">
+        <is>
+          <t>Streamed (SSE/NDJSON): progress events → final stats (rows, columns, match rate, new columns added) + merge_history entry.</t>
+        </is>
+      </c>
+      <c r="G28" s="4" t="inlineStr">
+        <is>
+          <t>Streaming progress card. On completion: "Merge Complete" hero with stats, column quality table, data preview. "What's Next" options: Redo, Another merge, Run DQA.</t>
+        </is>
+      </c>
+      <c r="H28" s="4" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I28" s="4" t="inlineStr">
+        <is>
+          <t>MAX_ROW_MULTIPLIER = 1.02 (join ops). MIN_MATCH_RATE = 0.30 (warning threshold). CSV download chunk = fetchmany(2000).</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="100" customHeight="1">
+      <c r="A29" s="14" t="inlineStr">
+        <is>
+          <t>6. Merge</t>
+        </is>
+      </c>
+      <c r="B29" s="15" t="inlineStr">
+        <is>
           <t>Skip merge</t>
         </is>
       </c>
-      <c r="C27" s="5" t="inlineStr">
+      <c r="C29" s="5" t="inlineStr">
         <is>
           <t>User clicks "Skip merge" (if only one group or user wants to skip).</t>
         </is>
       </c>
-      <c r="D27" s="5" t="inlineStr">
+      <c r="D29" s="5" t="inlineStr">
         <is>
           <t>sessionId, baseGroupId.</t>
         </is>
       </c>
-      <c r="E27" s="5" t="inlineStr">
+      <c r="E29" s="5" t="inlineStr">
         <is>
           <t>Base group's data copied directly to final_merged + versioned table. Merge history updated.</t>
         </is>
       </c>
-      <c r="F27" s="5" t="inlineStr">
+      <c r="F29" s="5" t="inlineStr">
         <is>
           <t>final_merged table created from base.</t>
         </is>
       </c>
-      <c r="G27" s="5" t="inlineStr">
+      <c r="G29" s="5" t="inlineStr">
         <is>
           <t>When only one table exists: shows a friendly Nothing to Merge card explaining all files were combined in the Append step, with a prominent Continue to Next Step button. When multiple tables exist: a subtle Skip merge entirely link under the dropdowns. Both call POST /api/merge/skip to create the final_merged table.</t>
         </is>
       </c>
-      <c r="H27" s="5" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="I27" s="5" t="inlineStr">
+      <c r="H29" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I29" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="100" customHeight="1">
-      <c r="A28" s="16" t="inlineStr">
+    <row r="30" ht="100" customHeight="1">
+      <c r="A30" s="16" t="inlineStr">
         <is>
           <t>7. Merge Results</t>
         </is>
       </c>
-      <c r="B28" s="17" t="inlineStr">
+      <c r="B30" s="17" t="inlineStr">
         <is>
           <t>View merge history</t>
         </is>
       </c>
-      <c r="C28" s="4" t="inlineStr">
+      <c r="C30" s="4" t="inlineStr">
         <is>
           <t>User reviews merge results.</t>
         </is>
       </c>
-      <c r="D28" s="4" t="inlineStr">
+      <c r="D30" s="4" t="inlineStr">
         <is>
           <t>None.</t>
         </is>
       </c>
-      <c r="E28" s="4" t="inlineStr">
+      <c r="E30" s="4" t="inlineStr">
         <is>
           <t>No API call — data already in state.</t>
         </is>
       </c>
-      <c r="F28" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="G28" s="4" t="inlineStr">
+      <c r="F30" s="4" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="G30" s="4" t="inlineStr">
         <is>
           <t>"Merge Step Complete" hero. Merge history list (versions, timestamps, sources). Options: "Go Back to Merge" (Step 6), "Run Data Quality Assessment" (Step 8).</t>
         </is>
       </c>
-      <c r="H28" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="I28" s="4" t="inlineStr">
+      <c r="H30" s="4" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I30" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="100" customHeight="1">
-      <c r="A29" s="16" t="inlineStr">
+    <row r="31" ht="100" customHeight="1">
+      <c r="A31" s="16" t="inlineStr">
         <is>
           <t>7. Merge Results</t>
         </is>
       </c>
-      <c r="B29" s="17" t="inlineStr">
+      <c r="B31" s="17" t="inlineStr">
         <is>
           <t>Merge Outputs Panel</t>
         </is>
       </c>
-      <c r="C29" s="5" t="inlineStr">
+      <c r="C31" s="5" t="inlineStr">
         <is>
           <t>User opens floating "Merge Outputs" tab (available from Step 6+).</t>
         </is>
       </c>
-      <c r="D29" s="5" t="inlineStr">
+      <c r="D31" s="5" t="inlineStr">
         <is>
           <t>sessionId, version.</t>
         </is>
       </c>
-      <c r="E29" s="5" t="inlineStr">
+      <c r="E31" s="5" t="inlineStr">
         <is>
           <t>Downloads use CSV streaming from final_merged_v{n}.</t>
         </is>
       </c>
-      <c r="F29" s="5" t="inlineStr">
+      <c r="F31" s="5" t="inlineStr">
         <is>
           <t>CSV/XLSX file streams. ZIP for "Download All".</t>
         </is>
       </c>
-      <c r="G29" s="5" t="inlineStr">
+      <c r="G31" s="5" t="inlineStr">
         <is>
           <t>List of output versions with label, rows, cols, sources, timestamp. Per-version: Download CSV. Download All ZIP. Send to Normalizer. Send to Summarizer. Delete with confirm.</t>
         </is>
       </c>
-      <c r="H29" s="5" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="I29" s="5" t="inlineStr">
+      <c r="H31" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I31" s="5" t="inlineStr">
         <is>
           <t>CSV streaming chunk = fetchmany(2000). Transfer timeout = 120s. Normalizer default URL = http://localhost:5000 (FE: http://localhost:3003). Summarizer default URL = http://localhost:3005 (FE: http://localhost:3004).</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="100" customHeight="1">
-      <c r="A30" s="18" t="inlineStr">
+    <row r="32" ht="100" customHeight="1">
+      <c r="A32" s="18" t="inlineStr">
         <is>
           <t>8. DQA</t>
         </is>
       </c>
-      <c r="B30" s="19" t="inlineStr">
+      <c r="B32" s="19" t="inlineStr">
         <is>
           <t>Date Analysis</t>
         </is>
       </c>
-      <c r="C30" s="4" t="inlineStr">
-        <is>
-          <t>Runs automatically on entering Step 8 (if API key set). User can select different date columns from dropdown.</t>
-        </is>
-      </c>
-      <c r="D30" s="4" t="inlineStr">
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>Expand the Date Analysis panel. The selected date column name is always shown. If multiple date columns exist, use the dropdown to pick a different one — this triggers a fresh backend analysis for the new column.</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr">
         <is>
           <t>sessionId, apiKey, tableName (e.g. final_merged_v1), optional dateColumn.</t>
         </is>
       </c>
-      <c r="E30" s="4" t="inlineStr">
-        <is>
-          <t>Validates the table exists via _validate_table. If table missing, raises TableMissingError (returned as code: TABLE_MISSING, 404). If session DB gone, raises ValueError. Then runs date format detection and AI insights.</t>
-        </is>
-      </c>
-      <c r="F30" s="4" t="inlineStr">
+      <c r="E32" s="4" t="inlineStr">
+        <is>
+          <t>Uses column_resolver.py to find date columns via 3-tier matching (exact, alias, fuzzy) plus any column with date in the name. Detects date formats per file, builds year x month spend pivot, computes total spend summary. Spend parsing handles thousands separators (commas/spaces). AI insight uses consolidated financial prompt (1 LLM call for date+currency+payment terms) and returns exactly 3 structured bullet points.</t>
+        </is>
+      </c>
+      <c r="F32" s="4" t="inlineStr">
         <is>
           <t>formatTable (per-file format analysis), consistent flag, pivotData (year × month spend), aiInsight.</t>
         </is>
       </c>
-      <c r="G30" s="4" t="inlineStr">
-        <is>
-          <t>If TABLE_MISSING error code, shows Merge Data Not Found card with Back to Merge button. Otherwise shows date analysis panel with format distribution and AI insight.</t>
-        </is>
-      </c>
-      <c r="H30" s="4" t="inlineStr">
+      <c r="G32" s="4" t="inlineStr">
+        <is>
+          <t>AI insight, format table, spend pivot, and total spend summary. The column selector is always visible: as a dropdown when multiple columns exist, or as a label when only one was detected.</t>
+        </is>
+      </c>
+      <c r="H32" s="4" t="inlineStr">
         <is>
           <t>System: "You are a senior procurement data-quality consultant... payload includes formatTable, consistent, pivotData, selectedColumn... If inconsistent, state date normalisation required... If pivotData, analyse seasonality, YoY trends, data gaps, anomalies..."
 User: JSON payload with those fields.
 Response: {"insight": "- bullet1\n- bullet2\n..."}.</t>
         </is>
       </c>
-      <c r="I30" s="4" t="inlineStr">
+      <c r="I32" s="4" t="inlineStr">
         <is>
           <t>TRY_CAST instead of CAST for date extraction</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="100" customHeight="1">
-      <c r="A31" s="18" t="inlineStr">
+    <row r="33" ht="100" customHeight="1">
+      <c r="A33" s="18" t="inlineStr">
         <is>
           <t>8. DQA</t>
         </is>
       </c>
-      <c r="B31" s="19" t="inlineStr">
+      <c r="B33" s="19" t="inlineStr">
         <is>
           <t>Currency Analysis</t>
         </is>
       </c>
-      <c r="C31" s="5" t="inlineStr">
-        <is>
-          <t>Runs automatically alongside Date.</t>
-        </is>
-      </c>
-      <c r="D31" s="5" t="inlineStr">
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>Reviews the currency panel. Can change the analysis column via a dropdown (pre-filled by AI suggestion). Selecting a different column automatically reruns the currency analysis.</t>
+        </is>
+      </c>
+      <c r="D33" s="5" t="inlineStr">
         <is>
           <t>sessionId, apiKey, tableName.</t>
         </is>
       </c>
-      <c r="E31" s="5" t="inlineStr">
-        <is>
-          <t>Validates table via _validate_table (raises TableMissingError with code TABLE_MISSING if missing). Then runs currency quality analysis and AI insights.</t>
-        </is>
-      </c>
-      <c r="F31" s="5" t="inlineStr">
-        <is>
-          <t>currencyTable, distinctCount, codes, aiInsight.</t>
-        </is>
-      </c>
-      <c r="G31" s="5" t="inlineStr">
-        <is>
-          <t>If TABLE_MISSING, shows Merge Data Not Found card with Back to Merge button. Otherwise shows currency panel.</t>
-        </is>
-      </c>
-      <c r="H31" s="5" t="inlineStr">
+      <c r="E33" s="5" t="inlineStr">
+        <is>
+          <t>run_currency_analysis_sql accepts an optional currency_column override. Uses find_currency_columns (keyword match on curr) merged with AI suggestions to populate available columns. Returns distribution stats and the list of available currency columns.</t>
+        </is>
+      </c>
+      <c r="F33" s="5" t="inlineStr">
+        <is>
+          <t>Currency distribution table, chosen column name, availableCurrencyColumns list</t>
+        </is>
+      </c>
+      <c r="G33" s="5" t="inlineStr">
+        <is>
+          <t>AI insight shown prominently at top as 3 bullet points on soft blue background with amber left border. Currency table moved into collapsed View Details section. If no currency column found, shows empty state with muted icon.</t>
+        </is>
+      </c>
+      <c r="H33" s="5" t="inlineStr">
         <is>
           <t>System: "...currency quality analysis... Summarise distribution, flag standardisation needed, note non-standard codes, comment on local vs reporting spend..."
 User: JSON with currencyTable, distinctCount, codes.
 Response: {"insight": "..."}.</t>
         </is>
       </c>
-      <c r="I31" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="100" customHeight="1">
-      <c r="A32" s="18" t="inlineStr">
+      <c r="I33" s="5" t="inlineStr">
+        <is>
+          <t>currency_column (optional override from user dropdown)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="100" customHeight="1">
+      <c r="A34" s="18" t="inlineStr">
         <is>
           <t>8. DQA</t>
         </is>
       </c>
-      <c r="B32" s="19" t="inlineStr">
+      <c r="B34" s="19" t="inlineStr">
         <is>
           <t>Payment Terms Analysis</t>
         </is>
       </c>
-      <c r="C32" s="4" t="inlineStr">
-        <is>
-          <t>Runs automatically alongside Date.</t>
-        </is>
-      </c>
-      <c r="D32" s="4" t="inlineStr">
+      <c r="C34" s="4" t="inlineStr">
+        <is>
+          <t>Reviews the payment terms panel. Can change the analysis column via a dropdown (pre-filled by AI suggestion). Selecting a different column automatically reruns the payment terms analysis.</t>
+        </is>
+      </c>
+      <c r="D34" s="4" t="inlineStr">
         <is>
           <t>sessionId, apiKey, tableName.</t>
         </is>
       </c>
-      <c r="E32" s="4" t="inlineStr">
-        <is>
-          <t>Validates table via _validate_table (raises TableMissingError with code TABLE_MISSING if missing). Then runs payment terms analysis and AI insights.</t>
-        </is>
-      </c>
-      <c r="F32" s="4" t="inlineStr">
-        <is>
-          <t>paymentTerms, totalSpend, uniqueCount, aiInsight.</t>
-        </is>
-      </c>
-      <c r="G32" s="4" t="inlineStr">
-        <is>
-          <t>If TABLE_MISSING, shows Merge Data Not Found card with Back to Merge button. Otherwise shows payment terms panel.</t>
-        </is>
-      </c>
-      <c r="H32" s="4" t="inlineStr">
+      <c r="E34" s="4" t="inlineStr">
+        <is>
+          <t>run_payment_terms_analysis_sql accepts an optional payment_terms_column override. Uses find_payment_terms_columns (keyword match on payment/term) merged with AI suggestions to populate available columns. Returns distribution stats and the list of available payment terms columns.</t>
+        </is>
+      </c>
+      <c r="F34" s="4" t="inlineStr">
+        <is>
+          <t>Payment terms distribution table, chosen column name, availablePaymentTermsColumns list</t>
+        </is>
+      </c>
+      <c r="G34" s="4" t="inlineStr">
+        <is>
+          <t>AI insight at top as 3 bullet points on soft blue background with violet left border. Deep dive shows redesigned table with Term, Spend (Reporting), % of Rows, and per-currency spend columns if multiple currencies. If column not found, shows empty state.</t>
+        </is>
+      </c>
+      <c r="H34" s="4" t="inlineStr">
         <is>
           <t>System: "...payment terms analysis... Summarise distribution, identify standardisation scope (duplicates, variations like Net 30 / NET30 / Net-30), flag dominant/unusual terms, comment on working capital..."
 User: JSON with paymentTerms, totalSpend, uniqueCount.
 Response: {"insight": "..."}.</t>
         </is>
       </c>
-      <c r="I32" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="100" customHeight="1">
-      <c r="A33" s="18" t="inlineStr">
+      <c r="I34" s="4" t="inlineStr">
+        <is>
+          <t>payment_terms_column (optional override from user dropdown)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="100" customHeight="1">
+      <c r="A35" s="18" t="inlineStr">
         <is>
           <t>8. DQA</t>
         </is>
       </c>
-      <c r="B33" s="19" t="inlineStr">
+      <c r="B35" s="19" t="inlineStr">
         <is>
           <t>Country/Region Analysis</t>
         </is>
       </c>
-      <c r="C33" s="5" t="inlineStr">
+      <c r="C35" s="5" t="inlineStr">
         <is>
           <t>Runs automatically alongside Date.</t>
         </is>
       </c>
-      <c r="D33" s="5" t="inlineStr">
+      <c r="D35" s="5" t="inlineStr">
         <is>
           <t>sessionId, apiKey, tableName.</t>
         </is>
       </c>
-      <c r="E33" s="5" t="inlineStr">
-        <is>
-          <t>Validates table via _validate_table (raises TableMissingError with code TABLE_MISSING if missing). Then runs country/region analysis and AI insights.</t>
-        </is>
-      </c>
-      <c r="F33" s="5" t="inlineStr">
+      <c r="E35" s="5" t="inlineStr">
+        <is>
+          <t>Uses column_resolver.py find_country_columns to discover all country columns. Accepts a countryColumn parameter to let the user choose which column to analyse. Re-runs SQL and AI when the selection changes. AI insight uses consolidated entity prompt returning 3 structured bullet points for country and region separately.</t>
+        </is>
+      </c>
+      <c r="F35" s="5" t="inlineStr">
         <is>
           <t>countryValues, regionValues, countryColumn, regionColumn, countryInsight, regionInsight.</t>
         </is>
       </c>
-      <c r="G33" s="5" t="inlineStr">
-        <is>
-          <t>If TABLE_MISSING, shows Merge Data Not Found card with Back to Merge button. Otherwise shows country/region panel.</t>
-        </is>
-      </c>
-      <c r="H33" s="5" t="inlineStr">
+      <c r="G35" s="5" t="inlineStr">
+        <is>
+          <t>Country column dropdown at top for selecting which column to analyse (defaults to Vendor Country). AI insight below (country + region stacked) as 3 bullet points each on soft blue background with emerald left border. Deep dive shows country and region values in a clean grid layout instead of plain pills.</t>
+        </is>
+      </c>
+      <c r="H35" s="5" t="inlineStr">
         <is>
           <t>System: "...country and region data... For countries: check mixed formats (US vs United States vs USA), inconsistent casing, spelling variations, flag standardisation needed. For regions: same analysis..."
 User: JSON with countryValues, regionValues, column names.
 Response: {"countryInsight": "..." or null, "regionInsight": "..." or null}.</t>
         </is>
       </c>
-      <c r="I33" s="5" t="inlineStr">
+      <c r="I35" s="5" t="inlineStr">
         <is>
           <t>Country/region chips capped at 100 display + "+N more".</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="100" customHeight="1">
-      <c r="A34" s="18" t="inlineStr">
+    <row r="36" ht="100" customHeight="1">
+      <c r="A36" s="18" t="inlineStr">
         <is>
           <t>8. DQA</t>
         </is>
       </c>
-      <c r="B34" s="19" t="inlineStr">
+      <c r="B36" s="19" t="inlineStr">
         <is>
           <t>Supplier Analysis</t>
         </is>
       </c>
-      <c r="C34" s="4" t="inlineStr">
-        <is>
-          <t>Runs automatically alongside Date.</t>
-        </is>
-      </c>
-      <c r="D34" s="4" t="inlineStr">
+      <c r="C36" s="4" t="inlineStr">
+        <is>
+          <t>Reviews the supplier panel. Can change the analysis column via a dropdown (pre-filled by AI suggestion). Selecting a different column automatically reruns the supplier analysis.</t>
+        </is>
+      </c>
+      <c r="D36" s="4" t="inlineStr">
         <is>
           <t>sessionId, apiKey, tableName.</t>
         </is>
       </c>
-      <c r="E34" s="4" t="inlineStr">
-        <is>
-          <t>Fetches top suppliers by spend from the merged table. Sends the list to the AI with a short prompt requesting only 2-3 bullet points on whether normalisation is needed plus 2-3 example supplier name cases. No stat cards are shown.</t>
-        </is>
-      </c>
-      <c r="F34" s="4" t="inlineStr">
-        <is>
-          <t>Supplier names list, aiInsight.</t>
-        </is>
-      </c>
-      <c r="G34" s="4" t="inlineStr">
-        <is>
-          <t>Short AI insight banner with 2-3 bullet points (no stat cards).</t>
-        </is>
-      </c>
-      <c r="H34" s="4" t="inlineStr">
+      <c r="E36" s="4" t="inlineStr">
+        <is>
+          <t>run_supplier_analysis_sql accepts an optional vendor_column override. Uses find_supplier_columns (keyword match on vendor/supplier) merged with AI suggestions to populate available columns. Returns distribution stats and the list of available supplier columns.</t>
+        </is>
+      </c>
+      <c r="F36" s="4" t="inlineStr">
+        <is>
+          <t>Supplier distribution table, chosen column name, availableSupplierColumns list</t>
+        </is>
+      </c>
+      <c r="G36" s="4" t="inlineStr">
+        <is>
+          <t>AI insight at top as 3 bullet points on soft blue background with rose left border. If reporting spend exists, deep dive shows Pareto stat line and top 20 suppliers table. If no spend data, shows AI insight only with no deep dive.</t>
+        </is>
+      </c>
+      <c r="H36" s="4" t="inlineStr">
         <is>
           <t>System: "...list of supplier names sorted alphabetically, top suppliers by spend... Analyse for: potential duplicates (Amazon Inc / Amazon Co / AMAZON INC.), inconsistent formatting (Corp vs Corporation), noise in names, groups of related entities. State whether supplier name normalisation is required and estimate scope..."
 User: JSON with supplier names.
 Response: {"insight": "..."}.</t>
         </is>
       </c>
-      <c r="I34" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="100" customHeight="1">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>8. DQA</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>Fill Rate Summary</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>Expand the Fill Rate Summary panel (shown above all other panels)</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>Session ID, table name</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>For each column, counts non-null/non-empty rows and divides by total rows to get fill rate. For spend coverage, if reporting currency spend exists, computes spend-where-column-is-filled / total-spend. If only local spend, groups by currency code and computes per-currency percentage.</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>JSON with per-column pctRowsCovered, spendCoverage (single % or array of {code,pct}), spendType, spendColumn</t>
-        </is>
-      </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>Table with Column Name, % Rows Covered, and % of Total Spend (or % of Local Spend by Currency)</t>
-        </is>
-      </c>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="I35" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="100" customHeight="1">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>8. DQA</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>Total Spend Summary (Date panel)</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>View the summary block above the date-spend pivot table</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>Session ID, table name, date column</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>After building the pivot, sums spend. If reporting currency, returns a single total. If only local, groups by currency and returns per-currency totals.</t>
-        </is>
-      </c>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>totalSpendSummary field: {type: reporting, total} or {type: local_by_currency, currencies: [{code, total}]}</t>
-        </is>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>Summary line above pivot: single total or comma-separated currency totals (e.g. 965 USD, 765 EUR)</t>
-        </is>
-      </c>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="I36" t="inlineStr">
-        <is>
-          <t>NA</t>
+      <c r="I36" s="4" t="inlineStr">
+        <is>
+          <t>vendor_column (optional override from user dropdown)</t>
         </is>
       </c>
     </row>
@@ -2353,136 +2353,324 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
+          <t>Fill Rate Summary</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Expand the Fill Rate Summary panel (shown above all other panels)</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Session ID, table name</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Uses column_resolver.py for spend column detection. Fill rate calculation now excludes null-proxy values (N/A, unknown, null, etc.) giving an effective fill rate. Spend parsing handles thousands separators.</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>JSON with per-column pctRowsCovered, spendCoverage (single % or array of {code,pct}), spendType, spendColumn</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Table with zebra-striped rows showing column name, effective fill rate (excluding null proxies), and spend coverage. No AI insight for this panel.</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>8. DQA</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Total Spend Summary (Date panel)</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>View the summary block above the date-spend pivot table</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Session ID, table name, date column</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>After building the pivot, sums spend. If reporting currency, returns a single total. If only local, groups by currency and returns per-currency totals.</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>totalSpendSummary field: {type: reporting, total} or {type: local_by_currency, currencies: [{code, total}]}</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Summary line above pivot: single total or comma-separated currency totals (e.g. 965 USD, 765 EUR)</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>8. DQA</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
           <t>Spend Bifurcation</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="C39" t="inlineStr">
         <is>
           <t>Expand the Spend Bifurcation panel (shown after Date panel)</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr">
+      <c r="D39" t="inlineStr">
         <is>
           <t>Session ID, table name</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr">
+      <c r="E39" t="inlineStr">
         <is>
           <t>Identifies spend column (reporting currency first, then local). Sums positive and negative spend separately. If local, groups by currency code.</t>
         </is>
       </c>
-      <c r="F37" t="inlineStr">
+      <c r="F39" t="inlineStr">
         <is>
           <t>JSON with type (reporting/local/none), positiveSpend, negativeSpend, or currencies array with per-currency pos/neg totals</t>
         </is>
       </c>
-      <c r="G37" t="inlineStr">
+      <c r="G39" t="inlineStr">
         <is>
           <t>If reporting: two-column table with Total Positive Spend and Total Negative Spend. If local: three-column table with Currency, Total +ve Spend, Total -ve Spend.</t>
         </is>
       </c>
-      <c r="H37" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="I37" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="20" t="inlineStr">
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>8. DQA</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Consolidated DQA (all panels)</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Automatic when user lands on the DQA step</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Session ID, API key, table name, optional date/country column overrides</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>First calls collect_column_samples + suggest_columns_ai to get AI column suggestions (outside lock). Then runs all seven DQA panels in parallel via run_dqa_all_sql, passing AI-suggested columns as defaults for currency, payment terms, and supplier panels. Each panel returns its available columns list for dropdown population.</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>JSON dict keyed by panel name with complete results including AI insights as 3-element arrays</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>All DQA panels render together. Currency, Payment Terms, and Supplier panels each show a dropdown pre-filled with the AI-suggested column. User can switch columns in any dropdown to trigger a single-panel rerun.</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Two consolidated prompts: Financial Quality (date+currency+payment terms) and Entity Quality (country/region+supplier). Each returns structured 3-point insights per panel.</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>Fuzzy threshold: 0.75, max insight words: 10-15 per point</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>8. DQA</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>AI Column Suggestions</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>None ? runs automatically when the user starts the assessment</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>All column names from the working table plus 5 sample values per column, API key</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>collect_column_samples reads column names and samples under session lock. suggest_columns_ai sends them to the LLM outside the lock and returns the top-3 most likely columns per role (date, currency, payment_terms, country, vendor_name).</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>JSON dict keyed by role, each value a list of up to 3 column names ordered by confidence</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>No direct UI; the suggested columns pre-fill the default selections and dropdown options for each analysis panel</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>System prompt lists every role with a description. User prompt contains each column name with 5 sample values. LLM returns JSON mapping each role to an ordered array of top-3 column names.</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>sample_size=5 rows per column; model from call_ai_json config</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="20" t="inlineStr">
         <is>
           <t>Cross-cutting</t>
         </is>
       </c>
-      <c r="B38" s="21" t="inlineStr">
+      <c r="B42" s="21" t="inlineStr">
         <is>
           <t>Chat assistant</t>
         </is>
       </c>
-      <c r="C38" s="5" t="inlineStr">
+      <c r="C42" s="5" t="inlineStr">
         <is>
           <t>User opens chat panel and types a question at any step.</t>
         </is>
       </c>
-      <c r="D38" s="5" t="inlineStr">
+      <c r="D42" s="5" t="inlineStr">
         <is>
           <t>sessionId, message, context (auto-built from current stage, selected item, meta), apiKey, optional messages history.</t>
         </is>
       </c>
-      <c r="E38" s="5" t="inlineStr">
+      <c r="E42" s="5" t="inlineStr">
         <is>
           <t>System prompt defines the assistant as a procurement data expert embedded in DataStitcher. Context block injected with current stage data (counts, samples, groups, merge fields). Last 12 history messages included. Response is plain text (no JSON mode).</t>
         </is>
       </c>
-      <c r="F38" s="5" t="inlineStr">
+      <c r="F42" s="5" t="inlineStr">
         <is>
           <t>{content: "reply text"} via SSE (one message then [DONE]).</t>
         </is>
       </c>
-      <c r="G38" s="5" t="inlineStr">
+      <c r="G42" s="5" t="inlineStr">
         <is>
           <t>Chat panel with conversational AI assistant. Responds with procurement-aware advice, references actual column names and data from context.</t>
         </is>
       </c>
-      <c r="H38" s="5" t="inlineStr">
+      <c r="H42" s="5" t="inlineStr">
         <is>
           <t>System: "You are a concise data assistant embedded in DataStitcher, with deep expertise in procurement and supply chain data... Rules: be concise, 2-4 paragraphs max, plain language, reference actual column names... Procurement perspective: use procurement terminology (spend analysis, suppliers, categories, PO, invoices, contracts, OTIF, DPO, maverick spend, tail spend...)"
 User: The user's message.
 Context: Auto-built JSON with stage, meta, samples.</t>
         </is>
       </c>
-      <c r="I38" s="5" t="inlineStr">
+      <c r="I42" s="5" t="inlineStr">
         <is>
           <t>Last 12 history messages. AI cache TTL = 300s. AI retry attempts = 3.</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="20" t="inlineStr">
+    <row r="43">
+      <c r="A43" s="20" t="inlineStr">
         <is>
           <t>Cross-cutting</t>
         </is>
       </c>
-      <c r="B39" s="21" t="inlineStr">
+      <c r="B43" s="21" t="inlineStr">
         <is>
           <t>Group Insights (pipeline)</t>
         </is>
       </c>
-      <c r="C39" s="4" t="inlineStr">
+      <c r="C43" s="4" t="inlineStr">
         <is>
           <t>Currently not exposed in UI — backend-only pipeline.</t>
         </is>
       </c>
-      <c r="D39" s="4" t="inlineStr">
+      <c r="D43" s="4" t="inlineStr">
         <is>
           <t>sessionId, apiKey, groupIds.</t>
         </is>
       </c>
-      <c r="E39" s="4" t="inlineStr">
+      <c r="E43" s="4" t="inlineStr">
         <is>
           <t>Multi-step AI pipeline per group: (1) Data Profiler — column stats → data description, column roles, domain keywords. (2) Quality Auditor — scores quality 0–100, identifies issues by severity, recommends fixes. (3) Analytics Strategist — suggests up to 5 slices (GROUP BY dimension + aggregation). SQL executed for each slice (LIMIT 15 rows). (4) Insight Synthesizer — combines everything into top 3–5 findings with specific numbers. Cross-group: Cross-Group Synthesizer — narrative about how groups relate, merge hints.</t>
         </is>
       </c>
-      <c r="F39" s="4" t="inlineStr">
+      <c r="F43" s="4" t="inlineStr">
         <is>
           <t>Per-group: summary, topInsights, suggestedActions, qualityScore, issues. Cross-group: narrative, mergeHints.</t>
         </is>
       </c>
-      <c r="G39" s="4" t="inlineStr">
+      <c r="G43" s="4" t="inlineStr">
         <is>
           <t>Not rendered in current UI.</t>
         </is>
       </c>
-      <c r="H39" s="4" t="inlineStr">
+      <c r="H43" s="4" t="inlineStr">
         <is>
           <t>Profiler, Auditor, Strategist, Synthesizer, Cross-Group Synthesizer — each has a dedicated system prompt (see insight prompt chain). All return structured JSON.</t>
         </is>
       </c>
-      <c r="I39" s="4" t="inlineStr">
+      <c r="I43" s="4" t="inlineStr">
         <is>
           <t>Strategist slices capped at 5. Slice SQL LIMIT 15. Cross-group value overlap slice = 15. AI pool workers up to 6.</t>
         </is>
@@ -2501,7 +2689,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H24"/>
+  <dimension ref="A1:H32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -3001,26 +3189,22 @@
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>Calls run_executive_summary() which runs four analyses: (1) Date-spend pivot via SQL with non-numeric spend excluded, (2) Spend bifurcation (positive vs negative), (3) Pareto analysis using pandas -- groups by supplier, sums positive spend per supplier, sorts descending, computes cumulative %, then counts invoice rows and unique transaction types for suppliers at each threshold (80/85/90/95/99%), (4) Description quality with AI. Negative spend and credit notes are excluded from Pareto ranking.</t>
+          <t>run_executive_summary_sql() computes all panels: date pivot, spend bifurcation (with negPctOfPos, negRowCount, netSpend), Pareto analysis (80/85/90/95%%), date period, spend breakdown, supplier breakdown, categorization effort, flags, column fill rate, description quality stats. run_executive_summary_ai() then calls _generate_categorization_recommendation() for the AI method recommendation.</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>totalRows, datePivot (month×year spend grid), paretoAnalysis (threshold breakdowns), descriptionQuality[] (per-column stats + AI aiInsight).</t>
+          <t>JSON with datePeriod, spendBreakdown, supplierBreakdown, categorizationEffort (with AI buckets/verdict/method/cost), flags, columnFillRate, datePivot, spendBifurcation, paretoAnalysis, descriptionQuality, totalRows</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>(1) Date Spend Pivot table (month × year).
-(2) Spend &amp; Supplier Analysis with Pareto thresholds (80–99%) showing total spend, transaction counts, supplier counts.
-(3) Description Quality per column with spend covered, expandable Top 10 most frequent descriptions, and an AI-generated quality insight in bullet points.</t>
+          <t>Executive Summary panel with one-liner statements (date range, LTM spend, supplier count, categorization recommendation + cost), conditional flag bullets (amber/red), plus collapsible panels for Column Fill Rate, Negative vs Positive Spend, Year/Monthly Spend Split, and Pareto Cuts (80/85/90/95)</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>System: "You are a senior procurement data-quality consultant... You will receive a JSON payload containing: descriptionType, sampledDescriptions (up to 100 from top 80% spend), topByFrequency (100 most common with count+spend), backendStats (avgLength, multiWordCount/Spend, nullProxyCount/Spend, totalPopulated, totalSpend)... Produce 5–8 bullets on clarity, content type, languages, categorisation suitability, null-proxy quality, multi-word split, overall verdict."
-User: JSON with those 4 keys.
-Response: {"insight": "- bullet1\n- bullet2\n..."}.</t>
+          <t>CATEGORIZATION_EFFORT_PROMPT: analyses top 1000 descriptions, buckets them into high/medium/low quality, returns qualityVerdict, recommendedMethod (MapAI or Creactives), and reasoning citing the pre-computed MapAI cost. Python rule engine overrides: forces Creactives when row_count &gt; 400K.</t>
         </is>
       </c>
     </row>
@@ -3067,168 +3251,504 @@
       </c>
     </row>
     <row r="14" ht="90" customHeight="1">
-      <c r="A14" s="12" t="inlineStr">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>4. Spend Quality Assessment</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Not Procurable Spend keyword search</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>User switches to the Not Procurable Spend tab, selects one or more description columns from pill-shaped toggles, types a keyword in the search bar, and presses Enter or clicks Add. Each keyword appears in a results table with matching row count and total spend. User can remove keywords by clicking the trash icon or the X on keyword chips.</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Session ID, selected column field keys (e.g. description, po_material_description, l1-l4, supplier), keyword string</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Two endpoints: POST /not-procurable/columns queries information_schema.columns for analysis_data and returns the subset of string-type columns that are searchable. POST /not-procurable/search builds a DuckDB query with ILIKE clauses across all selected columns and returns COUNT(*) and SUM(total_spend) for matching rows. Keywords are SQL-escaped to prevent injection.</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>columns endpoint: {columns: [{fieldKey, displayName}]}. search endpoint: {keyword, matchingRows, totalSpend}</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>A tab bar with Executive Summary and Not Procurable Spend tabs. The Not Procurable Spend tab shows a column selector with pill toggles, a keyword search bar with Add button, keyword chips, and a results table with Keyword, Matching Rows, Total Spend columns plus a bold Totals footer row.</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="90" customHeight="1">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>4. Spend Quality Assessment</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Intercompany Spend keyword search</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>User switches to the Intercompany Spend tab, selects vendor columns (pills), types keywords and presses Enter to search</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Session ID, selected vendor column fieldKeys, keyword string</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>get_vendor_searchable_columns() returns vendor columns present in analysis_data. search_intercompany_keyword() runs ILIKE search across selected vendor columns and sums total_spend for matching rows.</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>JSON with columns list or keyword match result {keyword, matchingRows, totalSpend}</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Intercompany Spend tab with column selector pills, keyword search input, keyword chips, and results table showing per-keyword row count and spend with a total row</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="90" customHeight="1">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>4. Spend Quality Assessment</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Date period analysis</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>None ? runs automatically</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>invoice_date column from analysis_data</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>_compute_date_period() finds MIN/MAX of invoice_date, formats period label, counts distinct year-month combos</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Dict with startDate, endDate, periodLabel, monthsCovered, feasible flag</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Period label displayed in Executive Summary header area</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="90" customHeight="1">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>4. Spend Quality Assessment</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Spend breakdown (LTM + FY)</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>None ? runs automatically</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>total_spend and invoice_date columns from analysis_data</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>_compute_spend_breakdown() computes LTM spend (12 months to max date), current/prior FY spend, and YoY change</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Dict with ltmSpend, currentFySpend, priorFySpend, yoyAbs, yoyPct, FY labels, feasible flag</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Spend breakdown panel in Executive Summary showing LTM, FY figures, and YoY delta</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="90" customHeight="1">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>4. Spend Quality Assessment</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Supplier breakdown</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>None ? runs automatically</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>supplier and total_spend columns from analysis_data</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>_compute_supplier_breakdown() groups by supplier, computes 80%% threshold, top-10, and duplicate name detection via case-insensitive matching</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Dict with totalSuppliers, suppliersTo80Pct, top10 list, duplicateNameFlags count, feasible flag</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Supplier breakdown panel showing counts, top-10 table, and duplicate warnings</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="90" customHeight="1">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>4. Spend Quality Assessment</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Categorization effort estimate</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>None ? runs automatically (AI phase adds recommendation)</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>description column (+ supplier, total_spend if available) from analysis_data</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>_compute_categorization_effort() computes avgWordCount, avgCharLength, fillRate, uniqueCount, distinctPairs; estimates AI cost using GPT token rates. AI phase calls _generate_categorization_recommendation() for method recommendation.</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Dict with metrics, mapAICost, forcedMethod, top1000Descriptions, buckets, qualityVerdict, recommendedMethod, reasoning, feasible flag</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Categorization effort panel showing description stats, estimated cost, and AI-recommended method (MapAI vs Creactives)</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>CATEGORIZATION_RECOMMENDATION_PROMPT: asks AI to bucket descriptions into high/medium/low quality tiers, give a verdict, and recommend MapAI or Creactives with reasoning</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="90" customHeight="1">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>4. Spend Quality Assessment</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Quality flags</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>None ? runs automatically</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>date_pivot cells, description/supplier/priority columns from analysis_data</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>_compute_flags() checks spend consistency (months &gt;20%% from average), description quality (fill &lt;70%% or words &lt;2), vendor quality (fill &lt;75%%), and null columns (fill &lt;80%% or spend coverage &lt;90%%)</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Dict with spendConsistency, descriptionQuality, vendorQuality, nullColumns ? each None or a details dict</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Flags panel highlighting data quality issues with specific metrics and affected months/columns</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="90" customHeight="1">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>4. Spend Quality Assessment</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Column fill rate table</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>None ? runs automatically</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>All mapped columns from analysis_data plus total_spend for coverage calc</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>_compute_column_fill_rate() iterates every column, computes fill rate (non-null non-empty / total) and spend coverage (spend in populated rows / total spend). Sorted by spend coverage desc.</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Dict with columns list (columnName, fillRate, spendCoverage) and feasible flag</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Column fill rate table showing every column with fill percentage and spend coverage percentage</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="90" customHeight="1">
+      <c r="A22" s="12" t="inlineStr">
         <is>
           <t>5. Select Views</t>
         </is>
       </c>
-      <c r="B14" s="13" t="inlineStr">
+      <c r="B22" s="13" t="inlineStr">
         <is>
           <t>Check available views</t>
         </is>
       </c>
-      <c r="C14" s="5" t="inlineStr">
+      <c r="C22" s="5" t="inlineStr">
         <is>
           <t>No user action — available views are fetched right after confirming mapping in Step 3.</t>
         </is>
       </c>
-      <c r="D14" s="5" t="inlineStr">
+      <c r="D22" s="5" t="inlineStr">
         <is>
           <t>The confirmed mapping object.</t>
         </is>
       </c>
-      <c r="E14" s="5" t="inlineStr">
+      <c r="E22" s="5" t="inlineStr">
         <is>
           <t>Each of the 9 dashboard views in VIEW_REGISTRY is checked: does the mapping include all its requiredFields? (e.g. Spend Over Time needs invoice_date + total_spend).</t>
         </is>
       </c>
-      <c r="F14" s="5" t="inlineStr">
+      <c r="F22" s="5" t="inlineStr">
         <is>
           <t>List of 9 views with available: true/false per view.</t>
         </is>
       </c>
-      <c r="G14" s="5" t="inlineStr">
+      <c r="G22" s="5" t="inlineStr">
         <is>
           <t>Grid of view cards: available ones have checkboxes (default on), unavailable ones are dimmed with a lock icon and "Missing columns" note.</t>
         </is>
       </c>
-      <c r="H14" s="5" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="90" customHeight="1">
-      <c r="A15" s="12" t="inlineStr">
+      <c r="H22" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="90" customHeight="1">
+      <c r="A23" s="12" t="inlineStr">
         <is>
           <t>5. Select Views</t>
         </is>
       </c>
-      <c r="B15" s="13" t="inlineStr">
+      <c r="B23" s="13" t="inlineStr">
         <is>
           <t>Select and generate views</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="C23" s="4" t="inlineStr">
         <is>
           <t>User toggles checkboxes for the views they want, then clicks "Generate Views".</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr">
+      <c r="D23" s="4" t="inlineStr">
         <is>
           <t>List of selected viewIds + config (empty by default).</t>
         </is>
       </c>
-      <c r="E15" s="4" t="inlineStr">
+      <c r="E23" s="4" t="inlineStr">
         <is>
           <t>For each selected view, pandas aggregations run against analysis_data: groupby, sum, sort, cumulative calculations, etc. Metrics are extracted (e.g. total spend, top supplier %, date range). Results stored in view_results in the DB.</t>
         </is>
       </c>
-      <c r="F15" s="4" t="inlineStr">
+      <c r="F23" s="4" t="inlineStr">
         <is>
           <t>Per view: tableData (aggregated rows), chartData (formatted for charts), metrics (key numbers), chartType.</t>
         </is>
       </c>
-      <c r="G15" s="4" t="inlineStr">
+      <c r="G23" s="4" t="inlineStr">
         <is>
           <t>User advances to Step 6 (Dashboard). In parallel, if API key is set, AI summaries are triggered for each computed view (except category_drilldown).</t>
         </is>
       </c>
-      <c r="H15" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="90" customHeight="1">
-      <c r="A16" s="14" t="inlineStr">
+      <c r="H23" s="4" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="14" t="inlineStr">
         <is>
           <t>6. Dashboard</t>
         </is>
       </c>
-      <c r="B16" s="15" t="inlineStr">
+      <c r="B24" s="15" t="inlineStr">
         <is>
           <t>View charts and tables</t>
         </is>
       </c>
-      <c r="C16" s="5" t="inlineStr">
+      <c r="C24" s="5" t="inlineStr">
         <is>
           <t>User views the dashboard with all computed views.</t>
         </is>
       </c>
-      <c r="D16" s="5" t="inlineStr">
+      <c r="D24" s="5" t="inlineStr">
         <is>
           <t>Computed view results from Step 5.</t>
         </is>
       </c>
-      <c r="E16" s="5" t="inlineStr">
+      <c r="E24" s="5" t="inlineStr">
         <is>
           <t>View engine loads analysis_data and explicitly coerces known string columns (supplier_name, currency_code, etc.) to str and numeric columns (total_spend) to pd.to_numeric. All percentage-of-total calculations use max(total, 1e-9) to prevent division by zero. Datetime column detection uses pd.api.types.is_datetime64_any_dtype for robustness.</t>
         </is>
       </c>
-      <c r="F16" s="5" t="inlineStr">
+      <c r="F24" s="5" t="inlineStr">
         <is>
           <t>None (already computed).</t>
         </is>
       </c>
-      <c r="G16" s="5" t="inlineStr">
+      <c r="G24" s="5" t="inlineStr">
         <is>
           <t>Each view shows as a collapsible panel with: a chart (bar, horizontal bar, pareto, or mekko), an AI Analysis sidebar with markdown summary, and a toggle to show the underlying data table. Export CSV button per view.</t>
         </is>
       </c>
-      <c r="H16" s="5" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="90" customHeight="1">
-      <c r="A17" s="14" t="inlineStr">
+      <c r="H24" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="14" t="inlineStr">
         <is>
           <t>6. Dashboard</t>
         </is>
       </c>
-      <c r="B17" s="15" t="inlineStr">
+      <c r="B25" s="15" t="inlineStr">
         <is>
           <t>Generate AI summary</t>
         </is>
       </c>
-      <c r="C17" s="4" t="inlineStr">
+      <c r="C25" s="4" t="inlineStr">
         <is>
           <t>Runs automatically after views are computed (if API key is set). User can re-trigger from the dashboard.</t>
         </is>
       </c>
-      <c r="D17" s="4" t="inlineStr">
+      <c r="D25" s="4" t="inlineStr">
         <is>
           <t>View's tableData (first 50 rows), chartType, metrics, plus optional pareto/drilldown fields.</t>
         </is>
       </c>
-      <c r="E17" s="4" t="inlineStr">
+      <c r="E25" s="4" t="inlineStr">
         <is>
           <t>The first 50 rows of the view's table data + metrics + chart type are sent to the LLM. A view-specific prompt focuses the AI on relevant aspects (e.g. trend for spend_over_time, concentration for supplier_ranking).</t>
         </is>
       </c>
-      <c r="F17" s="4" t="inlineStr">
+      <c r="F25" s="4" t="inlineStr">
         <is>
           <t>{"summary": "markdown text"} — stored in view_results[].aiSummary.</t>
         </is>
       </c>
-      <c r="G17" s="4" t="inlineStr">
+      <c r="G25" s="4" t="inlineStr">
         <is>
           <t>AI Analysis panel shows the markdown summary (bold numbers, bullet points, section headings). Skeleton loader shown while generating. category_drilldown gets no AI summary.</t>
         </is>
       </c>
-      <c r="H17" s="4" t="inlineStr">
+      <c r="H25" s="4" t="inlineStr">
         <is>
           <t>System: "You are a procurement analyst... write a concise analytical summary using clean markdown... bold for key figures... 3-5 bullets per section, 2-3 sections max." + view-specific focus (e.g. for spend_over_time: "Focus on: total spend, avg monthly, highest/lowest months, trend, spikes/dips").
 User: JSON payload with viewTitle, chartType, metrics, rowCount, columns, data (≤50 rows).
@@ -3236,295 +3756,295 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="90" customHeight="1">
-      <c r="A18" s="14" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="14" t="inlineStr">
         <is>
           <t>6. Dashboard</t>
         </is>
       </c>
-      <c r="B18" s="15" t="inlineStr">
+      <c r="B26" s="15" t="inlineStr">
         <is>
           <t>Adjust Pareto threshold</t>
         </is>
       </c>
-      <c r="C18" s="5" t="inlineStr">
+      <c r="C26" s="5" t="inlineStr">
         <is>
           <t>User moves the Pareto threshold slider (50–95%).</t>
         </is>
       </c>
-      <c r="D18" s="5" t="inlineStr">
+      <c r="D26" s="5" t="inlineStr">
         <is>
           <t>New threshold value + sessionId + viewId.</t>
         </is>
       </c>
-      <c r="E18" s="5" t="inlineStr">
+      <c r="E26" s="5" t="inlineStr">
         <is>
           <t>The Pareto view is recomputed from analysis_data with the new threshold — recalculates cumulative spend cutoff and which suppliers fall inside/outside.</t>
         </is>
       </c>
-      <c r="F18" s="5" t="inlineStr">
+      <c r="F26" s="5" t="inlineStr">
         <is>
           <t>Updated single view object merged into view_results.</t>
         </is>
       </c>
-      <c r="G18" s="5" t="inlineStr">
+      <c r="G26" s="5" t="inlineStr">
         <is>
           <t>Pareto chart and data table refresh. Supplier-in-group badge updates. Dashboard refreshes for that panel only.</t>
         </is>
       </c>
-      <c r="H18" s="5" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="90" customHeight="1">
-      <c r="A19" s="14" t="inlineStr">
+      <c r="H26" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="14" t="inlineStr">
         <is>
           <t>6. Dashboard</t>
         </is>
       </c>
-      <c r="B19" s="15" t="inlineStr">
+      <c r="B27" s="15" t="inlineStr">
         <is>
           <t>Adjust Top N suppliers</t>
         </is>
       </c>
-      <c r="C19" s="4" t="inlineStr">
+      <c r="C27" s="4" t="inlineStr">
         <is>
           <t>User moves the Top N slider (5–50) for the supplier ranking view.</t>
         </is>
       </c>
-      <c r="D19" s="4" t="inlineStr">
+      <c r="D27" s="4" t="inlineStr">
         <is>
           <t>New Top N value + sessionId + viewId.</t>
         </is>
       </c>
-      <c r="E19" s="4" t="inlineStr">
+      <c r="E27" s="4" t="inlineStr">
         <is>
           <t>The supplier ranking is recomputed from analysis_data with the new Top N — re-sorts and slices.</t>
         </is>
       </c>
-      <c r="F19" s="4" t="inlineStr">
+      <c r="F27" s="4" t="inlineStr">
         <is>
           <t>Updated single view object merged into view_results.</t>
         </is>
       </c>
-      <c r="G19" s="4" t="inlineStr">
+      <c r="G27" s="4" t="inlineStr">
         <is>
           <t>Supplier ranking chart and table refresh with the new top N. Dashboard refreshes for that panel only.</t>
         </is>
       </c>
-      <c r="H19" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="90" customHeight="1">
-      <c r="A20" s="14" t="inlineStr">
+      <c r="H27" s="4" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="14" t="inlineStr">
         <is>
           <t>6. Dashboard</t>
         </is>
       </c>
-      <c r="B20" s="15" t="inlineStr">
+      <c r="B28" s="15" t="inlineStr">
         <is>
           <t>Filter L1 for L2 vs L3 mekko</t>
         </is>
       </c>
-      <c r="C20" s="5" t="inlineStr">
+      <c r="C28" s="5" t="inlineStr">
         <is>
           <t>User selects an L1 category from the dropdown filter.</t>
         </is>
       </c>
-      <c r="D20" s="5" t="inlineStr">
+      <c r="D28" s="5" t="inlineStr">
         <is>
           <t>Selected L1 value + sessionId + viewId.</t>
         </is>
       </c>
-      <c r="E20" s="5" t="inlineStr">
+      <c r="E28" s="5" t="inlineStr">
         <is>
           <t>The L2 vs L3 mekko is recomputed filtering analysis_data to only the selected L1 category.</t>
         </is>
       </c>
-      <c r="F20" s="5" t="inlineStr">
+      <c r="F28" s="5" t="inlineStr">
         <is>
           <t>Updated single view object merged into view_results.</t>
         </is>
       </c>
-      <c r="G20" s="5" t="inlineStr">
+      <c r="G28" s="5" t="inlineStr">
         <is>
           <t>Mekko chart and table update to show only L2/L3 breakdown within the selected L1.</t>
         </is>
       </c>
-      <c r="H20" s="5" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="90" customHeight="1">
-      <c r="A21" s="14" t="inlineStr">
+      <c r="H28" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="14" t="inlineStr">
         <is>
           <t>6. Dashboard</t>
         </is>
       </c>
-      <c r="B21" s="15" t="inlineStr">
+      <c r="B29" s="15" t="inlineStr">
         <is>
           <t>Export CSV</t>
         </is>
       </c>
-      <c r="C21" s="4" t="inlineStr">
+      <c r="C29" s="4" t="inlineStr">
         <is>
           <t>User clicks the CSV export button on any view.</t>
         </is>
       </c>
-      <c r="D21" s="4" t="inlineStr">
+      <c r="D29" s="4" t="inlineStr">
         <is>
           <t>sessionId + viewId.</t>
         </is>
       </c>
-      <c r="E21" s="4" t="inlineStr">
+      <c r="E29" s="4" t="inlineStr">
         <is>
           <t>The stored view_results for that view is read. The first list found in tableData (prefers monthly/last12/yearly keys for multi-part views) is converted to CSV.</t>
         </is>
       </c>
-      <c r="F21" s="4" t="inlineStr">
+      <c r="F29" s="4" t="inlineStr">
         <is>
           <t>A CSV file stream.</t>
         </is>
       </c>
-      <c r="G21" s="4" t="inlineStr">
+      <c r="G29" s="4" t="inlineStr">
         <is>
           <t>Browser downloads a .csv file of the view's table data.</t>
         </is>
       </c>
-      <c r="H21" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="90" customHeight="1">
-      <c r="A22" s="16" t="inlineStr">
+      <c r="H29" s="4" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="16" t="inlineStr">
         <is>
           <t>7. Analysis Feasibility</t>
         </is>
       </c>
-      <c r="B22" s="17" t="inlineStr">
+      <c r="B30" s="17" t="inlineStr">
         <is>
           <t>Check Spend X-ray and Category Navigator feasibility</t>
         </is>
       </c>
-      <c r="C22" s="5" t="inlineStr">
+      <c r="C30" s="5" t="inlineStr">
         <is>
           <t>User switches between two tabs: Spend X-ray Analysis (24 dashboards) and Category Navigator Levers (14 levers). Each tab shows which items are feasible (green check) and which are not (with missing fields listed).</t>
         </is>
       </c>
-      <c r="D22" s="5" t="inlineStr">
+      <c r="D30" s="5" t="inlineStr">
         <is>
           <t>sessionId (the confirmed mapping is read from the DB).</t>
         </is>
       </c>
-      <c r="E22" s="5" t="inlineStr">
+      <c r="E30" s="5" t="inlineStr">
         <is>
           <t>get_procurement_view_availability checks both SPEND_XRAY_REGISTRY and CATEGORY_NAVIGATOR_REGISTRY against mapped field keys. Returns {spendXray: [...], categoryNavigator: [...]} with available flag and missingFields per entry.</t>
         </is>
       </c>
-      <c r="F22" s="5" t="inlineStr">
+      <c r="F30" s="5" t="inlineStr">
         <is>
           <t>{spendXray: [{viewId, title, available, missingFields}], categoryNavigator: [{viewId, title, available, missingFields}]}</t>
         </is>
       </c>
-      <c r="G22" s="5" t="inlineStr">
+      <c r="G30" s="5" t="inlineStr">
         <is>
           <t>Two-tab interface. Each tab shows a grid of feasibility cards with green check for feasible, red X for not feasible with missing field names listed.</t>
         </is>
       </c>
-      <c r="H22" s="5" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="90" customHeight="1">
-      <c r="A23" s="18" t="inlineStr">
+      <c r="H30" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="18" t="inlineStr">
         <is>
           <t>8. Email Generation</t>
         </is>
       </c>
-      <c r="B23" s="19" t="inlineStr">
+      <c r="B31" s="19" t="inlineStr">
         <is>
           <t>Fill context modal</t>
         </is>
       </c>
-      <c r="C23" s="4" t="inlineStr">
+      <c r="C31" s="4" t="inlineStr">
         <is>
           <t>User fills in: Recipient name, Client name, Sender name, Sender role, optional Scope note, and dynamic Next Steps rows (Action / Owner / Timeline).</t>
         </is>
       </c>
-      <c r="D23" s="4" t="inlineStr">
+      <c r="D31" s="4" t="inlineStr">
         <is>
           <t>User-entered context fields.</t>
         </is>
       </c>
-      <c r="E23" s="4" t="inlineStr">
+      <c r="E31" s="4" t="inlineStr">
         <is>
           <t>None — this is a frontend-only form. Context is assembled into an EmailContext object.</t>
         </is>
       </c>
-      <c r="F23" s="4" t="inlineStr">
+      <c r="F31" s="4" t="inlineStr">
         <is>
           <t>None.</t>
         </is>
       </c>
-      <c r="G23" s="4" t="inlineStr">
+      <c r="G31" s="4" t="inlineStr">
         <is>
           <t>A modal overlay with form fields for recipient, client, sender, role, scope, and a dynamic table for next steps. Non-empty next steps are included. User clicks "Generate Email" to submit.</t>
         </is>
       </c>
-      <c r="H23" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="18" t="inlineStr">
+      <c r="H31" s="4" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="18" t="inlineStr">
         <is>
           <t>8. Email Generation</t>
         </is>
       </c>
-      <c r="B24" s="19" t="inlineStr">
+      <c r="B32" s="19" t="inlineStr">
         <is>
           <t>Generate client email</t>
         </is>
       </c>
-      <c r="C24" s="5" t="inlineStr">
+      <c r="C32" s="5" t="inlineStr">
         <is>
           <t>User clicks "Generate Email" in the context modal.</t>
         </is>
       </c>
-      <c r="D24" s="5" t="inlineStr">
+      <c r="D32" s="5" t="inlineStr">
         <is>
           <t>Context from the form + all view metrics from view_results + API key.</t>
         </is>
       </c>
-      <c r="E24" s="5" t="inlineStr">
+      <c r="E32" s="5" t="inlineStr">
         <is>
           <t>View metrics are assembled into a structured JSON: each view's metrics are mapped to named sections (spend_vs_time, spend_vs_currency, spend_vs_country, supplier_ranking, pareto, spend_vs_l1, l1_vs_l2, l2_vs_l3). Context (names, scope, next_steps) is merged in. Missing views are flagged. This JSON + an email template are sent to the LLM.</t>
         </is>
       </c>
-      <c r="F24" s="5" t="inlineStr">
+      <c r="F32" s="5" t="inlineStr">
         <is>
           <t>{"email": "full email text", "subject": "subject line"} or {"error": "...", "fallback": "template-filled email"}.</t>
         </is>
       </c>
-      <c r="G24" s="5" t="inlineStr">
+      <c r="G32" s="5" t="inlineStr">
         <is>
           <t>An editable email view with subject field and body textarea. User can toggle Edit/Preview mode (markdown preview). Buttons: Copy to Clipboard, Regenerate, Back. On AI failure: amber error banner with Retry + "Use Template Fallback" button (fills body from a metrics-only template).</t>
         </is>
       </c>
-      <c r="H24" s="5" t="inlineStr">
+      <c r="H32" s="5" t="inlineStr">
         <is>
           <t>System: "You are a senior procurement consultant at a top-tier consulting firm. Using the view summaries below, write a professional client-facing spend data review email. Structure: 1) Opening 2) Spend Overview 3) Spend Trend 4) Supplier Landscape 5) Category Breakdown 6) Callouts 7) Next Steps. Tone: consulting style, lead with numbers, no filler. Auto-scale spend values. Return JSON: {email, subject}"
 User: "--- INPUT DATA ---\n" + pretty-printed JSON of assembled view metrics + context + "\n\n--- EMAIL TEMPLATE (use as a guide) ---\n" + a full example email template.

</xml_diff>

<commit_message>
merge step changes added
</commit_message>
<xml_diff>
--- a/.cursor/docs/FullAppDocumentation.xlsx
+++ b/.cursor/docs/FullAppDocumentation.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Module 1" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Module 3" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Module 2" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Module 1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Module 3" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Module 2" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Module 1'!$A$1:$I$36</definedName>
@@ -617,7 +617,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I43"/>
+  <dimension ref="A1:I45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1888,27 +1888,27 @@
       </c>
       <c r="E27" s="5" t="inlineStr">
         <is>
-          <t>Creates slim temp tables with only key + pull columns. Builds composite key as TRIM(LOWER(CAST(col AS TEXT))) joined with '|||'. Computes match rate, explosion factor, unmatched counts on both sides, duplicate key counts on source.</t>
+          <t>simulate_join() creates temp tables, runs SQL CTE with cardinality analysis (base_key_unique, source_key_unique, max rows per key), calculates match rates and explosion factor</t>
         </is>
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>matchRate, explosionFactor, unmatchedBase, unmatchedSource, duplicateSourceKeys.</t>
+          <t>JSON with match_rate, row_explosion_factor, unmatched counts, duplicate counts, key_cardinality (1:1/1:M/M:1/M:M), base_key_unique, source_key_unique, max rows per key</t>
         </is>
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>Simulation stats card: match rate %, explosion factor, unmatched rows on each side. Warnings if low match or high explosion.</t>
+          <t>7 stat cards including Key Relationship (colored cardinality badge), Match Rate, Row Explosion, etc.</t>
         </is>
       </c>
       <c r="H27" s="5" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="I27" s="5" t="inlineStr">
         <is>
-          <t>Composite key separator = '|||'. Debounce = 500 ms.</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -2007,435 +2007,435 @@
       </c>
     </row>
     <row r="30" ht="100" customHeight="1">
-      <c r="A30" s="16" t="inlineStr">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>6. Merge</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>AI Suggest Join Keys</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Click the AI Suggest Keys button after selecting base and source tables</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Base and source table metadata including column names and sample values</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Calls suggest_join_keys() which analyzes column match rates and queries AI with SYSTEM_PROMPT_SUGGEST_JOIN_KEYS</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>JSON array of suggested key pairs with confidence and reasoning</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Expandable panel showing 5-10 suggestions ranked by confidence with apply buttons</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>SYSTEM_PROMPT_SUGGEST_JOIN_KEYS - analyzes column metadata and match rates to suggest join key pairs</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>Sample size: 50-100 rows per column; Top matches: 20; Max suggestions returned: 5-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="100" customHeight="1">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>6. Merge</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Common columns reorder and highlight</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>View columns in side-by-side preview - common columns appear first with green badges</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Base and source columns, common column detection results</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Frontend getOrderedColumns() helper filters and sorts columns; renderTable() applies enhanced green styling</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>N/A - frontend only feature</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Columns reordered with common columns first, green Link2 badges, enhanced green backgrounds for common columns</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="100" customHeight="1">
+      <c r="A32" s="16" t="inlineStr">
         <is>
           <t>7. Merge Results</t>
         </is>
       </c>
-      <c r="B30" s="17" t="inlineStr">
+      <c r="B32" s="17" t="inlineStr">
         <is>
           <t>View merge history</t>
         </is>
       </c>
-      <c r="C30" s="4" t="inlineStr">
+      <c r="C32" s="4" t="inlineStr">
         <is>
           <t>User reviews merge results.</t>
         </is>
       </c>
-      <c r="D30" s="4" t="inlineStr">
+      <c r="D32" s="4" t="inlineStr">
         <is>
           <t>None.</t>
         </is>
       </c>
-      <c r="E30" s="4" t="inlineStr">
+      <c r="E32" s="4" t="inlineStr">
         <is>
           <t>No API call — data already in state.</t>
         </is>
       </c>
-      <c r="F30" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="G30" s="4" t="inlineStr">
+      <c r="F32" s="4" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="G32" s="4" t="inlineStr">
         <is>
           <t>"Merge Step Complete" hero. Merge history list (versions, timestamps, sources). Options: "Go Back to Merge" (Step 6), "Run Data Quality Assessment" (Step 8).</t>
         </is>
       </c>
-      <c r="H30" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="I30" s="4" t="inlineStr">
+      <c r="H32" s="4" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I32" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="100" customHeight="1">
-      <c r="A31" s="16" t="inlineStr">
+    <row r="33" ht="100" customHeight="1">
+      <c r="A33" s="16" t="inlineStr">
         <is>
           <t>7. Merge Results</t>
         </is>
       </c>
-      <c r="B31" s="17" t="inlineStr">
+      <c r="B33" s="17" t="inlineStr">
         <is>
           <t>Merge Outputs Panel</t>
         </is>
       </c>
-      <c r="C31" s="5" t="inlineStr">
+      <c r="C33" s="5" t="inlineStr">
         <is>
           <t>User opens floating "Merge Outputs" tab (available from Step 6+).</t>
         </is>
       </c>
-      <c r="D31" s="5" t="inlineStr">
+      <c r="D33" s="5" t="inlineStr">
         <is>
           <t>sessionId, version.</t>
         </is>
       </c>
-      <c r="E31" s="5" t="inlineStr">
+      <c r="E33" s="5" t="inlineStr">
         <is>
           <t>Downloads use CSV streaming from final_merged_v{n}.</t>
         </is>
       </c>
-      <c r="F31" s="5" t="inlineStr">
+      <c r="F33" s="5" t="inlineStr">
         <is>
           <t>CSV/XLSX file streams. ZIP for "Download All".</t>
         </is>
       </c>
-      <c r="G31" s="5" t="inlineStr">
+      <c r="G33" s="5" t="inlineStr">
         <is>
           <t>List of output versions with label, rows, cols, sources, timestamp. Per-version: Download CSV. Download All ZIP. Send to Normalizer. Send to Summarizer. Delete with confirm.</t>
         </is>
       </c>
-      <c r="H31" s="5" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="I31" s="5" t="inlineStr">
+      <c r="H33" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I33" s="5" t="inlineStr">
         <is>
           <t>CSV streaming chunk = fetchmany(2000). Transfer timeout = 120s. Normalizer default URL = http://localhost:5000 (FE: http://localhost:3003). Summarizer default URL = http://localhost:3005 (FE: http://localhost:3004).</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="100" customHeight="1">
-      <c r="A32" s="18" t="inlineStr">
+    <row r="34" ht="100" customHeight="1">
+      <c r="A34" s="18" t="inlineStr">
         <is>
           <t>8. DQA</t>
         </is>
       </c>
-      <c r="B32" s="19" t="inlineStr">
+      <c r="B34" s="19" t="inlineStr">
         <is>
           <t>Date Analysis</t>
         </is>
       </c>
-      <c r="C32" s="4" t="inlineStr">
+      <c r="C34" s="4" t="inlineStr">
         <is>
           <t>Expand the Date Analysis panel. The selected date column name is always shown. If multiple date columns exist, use the dropdown to pick a different one — this triggers a fresh backend analysis for the new column.</t>
         </is>
       </c>
-      <c r="D32" s="4" t="inlineStr">
+      <c r="D34" s="4" t="inlineStr">
         <is>
           <t>sessionId, apiKey, tableName (e.g. final_merged_v1), optional dateColumn.</t>
         </is>
       </c>
-      <c r="E32" s="4" t="inlineStr">
+      <c r="E34" s="4" t="inlineStr">
         <is>
           <t>Uses column_resolver.py to find date columns via 3-tier matching (exact, alias, fuzzy) plus any column with date in the name. Detects date formats per file, builds year x month spend pivot, computes total spend summary. Spend parsing handles thousands separators (commas/spaces). AI insight uses consolidated financial prompt (1 LLM call for date+currency+payment terms) and returns exactly 3 structured bullet points.</t>
         </is>
       </c>
-      <c r="F32" s="4" t="inlineStr">
+      <c r="F34" s="4" t="inlineStr">
         <is>
           <t>formatTable (per-file format analysis), consistent flag, pivotData (year × month spend), aiInsight.</t>
         </is>
       </c>
-      <c r="G32" s="4" t="inlineStr">
+      <c r="G34" s="4" t="inlineStr">
         <is>
           <t>AI insight, format table, spend pivot, and total spend summary. The column selector is always visible: as a dropdown when multiple columns exist, or as a label when only one was detected.</t>
         </is>
       </c>
-      <c r="H32" s="4" t="inlineStr">
+      <c r="H34" s="4" t="inlineStr">
         <is>
           <t>System: "You are a senior procurement data-quality consultant... payload includes formatTable, consistent, pivotData, selectedColumn... If inconsistent, state date normalisation required... If pivotData, analyse seasonality, YoY trends, data gaps, anomalies..."
 User: JSON payload with those fields.
 Response: {"insight": "- bullet1\n- bullet2\n..."}.</t>
         </is>
       </c>
-      <c r="I32" s="4" t="inlineStr">
+      <c r="I34" s="4" t="inlineStr">
         <is>
           <t>TRY_CAST instead of CAST for date extraction</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="100" customHeight="1">
-      <c r="A33" s="18" t="inlineStr">
+    <row r="35" ht="100" customHeight="1">
+      <c r="A35" s="18" t="inlineStr">
         <is>
           <t>8. DQA</t>
         </is>
       </c>
-      <c r="B33" s="19" t="inlineStr">
+      <c r="B35" s="19" t="inlineStr">
         <is>
           <t>Currency Analysis</t>
         </is>
       </c>
-      <c r="C33" s="5" t="inlineStr">
+      <c r="C35" s="5" t="inlineStr">
         <is>
           <t>Reviews the currency panel. Can change the analysis column via a dropdown (pre-filled by AI suggestion). Selecting a different column automatically reruns the currency analysis.</t>
         </is>
       </c>
-      <c r="D33" s="5" t="inlineStr">
+      <c r="D35" s="5" t="inlineStr">
         <is>
           <t>sessionId, apiKey, tableName.</t>
         </is>
       </c>
-      <c r="E33" s="5" t="inlineStr">
+      <c r="E35" s="5" t="inlineStr">
         <is>
           <t>run_currency_analysis_sql accepts an optional currency_column override. Uses find_currency_columns (keyword match on curr) merged with AI suggestions to populate available columns. Returns distribution stats and the list of available currency columns.</t>
         </is>
       </c>
-      <c r="F33" s="5" t="inlineStr">
+      <c r="F35" s="5" t="inlineStr">
         <is>
           <t>Currency distribution table, chosen column name, availableCurrencyColumns list</t>
         </is>
       </c>
-      <c r="G33" s="5" t="inlineStr">
+      <c r="G35" s="5" t="inlineStr">
         <is>
           <t>AI insight shown prominently at top as 3 bullet points on soft blue background with amber left border. Currency table moved into collapsed View Details section. If no currency column found, shows empty state with muted icon.</t>
         </is>
       </c>
-      <c r="H33" s="5" t="inlineStr">
+      <c r="H35" s="5" t="inlineStr">
         <is>
           <t>System: "...currency quality analysis... Summarise distribution, flag standardisation needed, note non-standard codes, comment on local vs reporting spend..."
 User: JSON with currencyTable, distinctCount, codes.
 Response: {"insight": "..."}.</t>
         </is>
       </c>
-      <c r="I33" s="5" t="inlineStr">
+      <c r="I35" s="5" t="inlineStr">
         <is>
           <t>currency_column (optional override from user dropdown)</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="100" customHeight="1">
-      <c r="A34" s="18" t="inlineStr">
+    <row r="36" ht="100" customHeight="1">
+      <c r="A36" s="18" t="inlineStr">
         <is>
           <t>8. DQA</t>
         </is>
       </c>
-      <c r="B34" s="19" t="inlineStr">
+      <c r="B36" s="19" t="inlineStr">
         <is>
           <t>Payment Terms Analysis</t>
         </is>
       </c>
-      <c r="C34" s="4" t="inlineStr">
+      <c r="C36" s="4" t="inlineStr">
         <is>
           <t>Reviews the payment terms panel. Can change the analysis column via a dropdown (pre-filled by AI suggestion). Selecting a different column automatically reruns the payment terms analysis.</t>
         </is>
       </c>
-      <c r="D34" s="4" t="inlineStr">
+      <c r="D36" s="4" t="inlineStr">
         <is>
           <t>sessionId, apiKey, tableName.</t>
         </is>
       </c>
-      <c r="E34" s="4" t="inlineStr">
+      <c r="E36" s="4" t="inlineStr">
         <is>
           <t>run_payment_terms_analysis_sql accepts an optional payment_terms_column override. Uses find_payment_terms_columns (keyword match on payment/term) merged with AI suggestions to populate available columns. Returns distribution stats and the list of available payment terms columns.</t>
         </is>
       </c>
-      <c r="F34" s="4" t="inlineStr">
+      <c r="F36" s="4" t="inlineStr">
         <is>
           <t>Payment terms distribution table, chosen column name, availablePaymentTermsColumns list</t>
         </is>
       </c>
-      <c r="G34" s="4" t="inlineStr">
+      <c r="G36" s="4" t="inlineStr">
         <is>
           <t>AI insight at top as 3 bullet points on soft blue background with violet left border. Deep dive shows redesigned table with Term, Spend (Reporting), % of Rows, and per-currency spend columns if multiple currencies. If column not found, shows empty state.</t>
         </is>
       </c>
-      <c r="H34" s="4" t="inlineStr">
+      <c r="H36" s="4" t="inlineStr">
         <is>
           <t>System: "...payment terms analysis... Summarise distribution, identify standardisation scope (duplicates, variations like Net 30 / NET30 / Net-30), flag dominant/unusual terms, comment on working capital..."
 User: JSON with paymentTerms, totalSpend, uniqueCount.
 Response: {"insight": "..."}.</t>
         </is>
       </c>
-      <c r="I34" s="4" t="inlineStr">
+      <c r="I36" s="4" t="inlineStr">
         <is>
           <t>payment_terms_column (optional override from user dropdown)</t>
         </is>
       </c>
     </row>
-    <row r="35" ht="100" customHeight="1">
-      <c r="A35" s="18" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="18" t="inlineStr">
         <is>
           <t>8. DQA</t>
         </is>
       </c>
-      <c r="B35" s="19" t="inlineStr">
+      <c r="B37" s="19" t="inlineStr">
         <is>
           <t>Country/Region Analysis</t>
         </is>
       </c>
-      <c r="C35" s="5" t="inlineStr">
+      <c r="C37" s="5" t="inlineStr">
         <is>
           <t>Runs automatically alongside Date.</t>
         </is>
       </c>
-      <c r="D35" s="5" t="inlineStr">
+      <c r="D37" s="5" t="inlineStr">
         <is>
           <t>sessionId, apiKey, tableName.</t>
         </is>
       </c>
-      <c r="E35" s="5" t="inlineStr">
+      <c r="E37" s="5" t="inlineStr">
         <is>
           <t>Uses column_resolver.py find_country_columns to discover all country columns. Accepts a countryColumn parameter to let the user choose which column to analyse. Re-runs SQL and AI when the selection changes. AI insight uses consolidated entity prompt returning 3 structured bullet points for country and region separately.</t>
         </is>
       </c>
-      <c r="F35" s="5" t="inlineStr">
+      <c r="F37" s="5" t="inlineStr">
         <is>
           <t>countryValues, regionValues, countryColumn, regionColumn, countryInsight, regionInsight.</t>
         </is>
       </c>
-      <c r="G35" s="5" t="inlineStr">
+      <c r="G37" s="5" t="inlineStr">
         <is>
           <t>Country column dropdown at top for selecting which column to analyse (defaults to Vendor Country). AI insight below (country + region stacked) as 3 bullet points each on soft blue background with emerald left border. Deep dive shows country and region values in a clean grid layout instead of plain pills.</t>
         </is>
       </c>
-      <c r="H35" s="5" t="inlineStr">
+      <c r="H37" s="5" t="inlineStr">
         <is>
           <t>System: "...country and region data... For countries: check mixed formats (US vs United States vs USA), inconsistent casing, spelling variations, flag standardisation needed. For regions: same analysis..."
 User: JSON with countryValues, regionValues, column names.
 Response: {"countryInsight": "..." or null, "regionInsight": "..." or null}.</t>
         </is>
       </c>
-      <c r="I35" s="5" t="inlineStr">
+      <c r="I37" s="5" t="inlineStr">
         <is>
           <t>Country/region chips capped at 100 display + "+N more".</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="100" customHeight="1">
-      <c r="A36" s="18" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="18" t="inlineStr">
         <is>
           <t>8. DQA</t>
         </is>
       </c>
-      <c r="B36" s="19" t="inlineStr">
+      <c r="B38" s="19" t="inlineStr">
         <is>
           <t>Supplier Analysis</t>
         </is>
       </c>
-      <c r="C36" s="4" t="inlineStr">
+      <c r="C38" s="4" t="inlineStr">
         <is>
           <t>Reviews the supplier panel. Can change the analysis column via a dropdown (pre-filled by AI suggestion). Selecting a different column automatically reruns the supplier analysis.</t>
         </is>
       </c>
-      <c r="D36" s="4" t="inlineStr">
+      <c r="D38" s="4" t="inlineStr">
         <is>
           <t>sessionId, apiKey, tableName.</t>
         </is>
       </c>
-      <c r="E36" s="4" t="inlineStr">
+      <c r="E38" s="4" t="inlineStr">
         <is>
           <t>run_supplier_analysis_sql accepts an optional vendor_column override. Uses find_supplier_columns (keyword match on vendor/supplier) merged with AI suggestions to populate available columns. Returns distribution stats and the list of available supplier columns.</t>
         </is>
       </c>
-      <c r="F36" s="4" t="inlineStr">
+      <c r="F38" s="4" t="inlineStr">
         <is>
           <t>Supplier distribution table, chosen column name, availableSupplierColumns list</t>
         </is>
       </c>
-      <c r="G36" s="4" t="inlineStr">
+      <c r="G38" s="4" t="inlineStr">
         <is>
           <t>AI insight at top as 3 bullet points on soft blue background with rose left border. If reporting spend exists, deep dive shows Pareto stat line and top 20 suppliers table. If no spend data, shows AI insight only with no deep dive.</t>
         </is>
       </c>
-      <c r="H36" s="4" t="inlineStr">
+      <c r="H38" s="4" t="inlineStr">
         <is>
           <t>System: "...list of supplier names sorted alphabetically, top suppliers by spend... Analyse for: potential duplicates (Amazon Inc / Amazon Co / AMAZON INC.), inconsistent formatting (Corp vs Corporation), noise in names, groups of related entities. State whether supplier name normalisation is required and estimate scope..."
 User: JSON with supplier names.
 Response: {"insight": "..."}.</t>
         </is>
       </c>
-      <c r="I36" s="4" t="inlineStr">
+      <c r="I38" s="4" t="inlineStr">
         <is>
           <t>vendor_column (optional override from user dropdown)</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>8. DQA</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>Fill Rate Summary</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>Expand the Fill Rate Summary panel (shown above all other panels)</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>Session ID, table name</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>Uses column_resolver.py for spend column detection. Fill rate calculation now excludes null-proxy values (N/A, unknown, null, etc.) giving an effective fill rate. Spend parsing handles thousands separators.</t>
-        </is>
-      </c>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>JSON with per-column pctRowsCovered, spendCoverage (single % or array of {code,pct}), spendType, spendColumn</t>
-        </is>
-      </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>Table with zebra-striped rows showing column name, effective fill rate (excluding null proxies), and spend coverage. No AI insight for this panel.</t>
-        </is>
-      </c>
-      <c r="H37" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="I37" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>8. DQA</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>Total Spend Summary (Date panel)</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>View the summary block above the date-spend pivot table</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>Session ID, table name, date column</t>
-        </is>
-      </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>After building the pivot, sums spend. If reporting currency, returns a single total. If only local, groups by currency and returns per-currency totals.</t>
-        </is>
-      </c>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t>totalSpendSummary field: {type: reporting, total} or {type: local_by_currency, currencies: [{code, total}]}</t>
-        </is>
-      </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>Summary line above pivot: single total or comma-separated currency totals (e.g. 965 USD, 765 EUR)</t>
-        </is>
-      </c>
-      <c r="H38" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="I38" t="inlineStr">
-        <is>
-          <t>NA</t>
         </is>
       </c>
     </row>
@@ -2447,12 +2447,12 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Spend Bifurcation</t>
+          <t>Fill Rate Summary</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Expand the Spend Bifurcation panel (shown after Date panel)</t>
+          <t>Expand the Fill Rate Summary panel (shown above all other panels)</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -2462,17 +2462,17 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Identifies spend column (reporting currency first, then local). Sums positive and negative spend separately. If local, groups by currency code.</t>
+          <t>Uses column_resolver.py for spend column detection. Fill rate calculation now excludes null-proxy values (N/A, unknown, null, etc.) giving an effective fill rate. Spend parsing handles thousands separators.</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>JSON with type (reporting/local/none), positiveSpend, negativeSpend, or currencies array with per-currency pos/neg totals</t>
+          <t>JSON with per-column pctRowsCovered, spendCoverage (single % or array of {code,pct}), spendType, spendColumn</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>If reporting: two-column table with Total Positive Spend and Total Negative Spend. If local: three-column table with Currency, Total +ve Spend, Total -ve Spend.</t>
+          <t>Table with zebra-striped rows showing column name, effective fill rate (excluding null proxies), and spend coverage. No AI insight for this panel.</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -2494,42 +2494,42 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Consolidated DQA (all panels)</t>
+          <t>Total Spend Summary (Date panel)</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Automatic when user lands on the DQA step</t>
+          <t>View the summary block above the date-spend pivot table</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Session ID, API key, table name, optional date/country column overrides</t>
+          <t>Session ID, table name, date column</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>First calls collect_column_samples + suggest_columns_ai to get AI column suggestions (outside lock). Then runs all seven DQA panels in parallel via run_dqa_all_sql, passing AI-suggested columns as defaults for currency, payment terms, and supplier panels. Each panel returns its available columns list for dropdown population.</t>
+          <t>After building the pivot, sums spend. If reporting currency, returns a single total. If only local, groups by currency and returns per-currency totals.</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>JSON dict keyed by panel name with complete results including AI insights as 3-element arrays</t>
+          <t>totalSpendSummary field: {type: reporting, total} or {type: local_by_currency, currencies: [{code, total}]}</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>All DQA panels render together. Currency, Payment Terms, and Supplier panels each show a dropdown pre-filled with the AI-suggested column. User can switch columns in any dropdown to trigger a single-panel rerun.</t>
+          <t>Summary line above pivot: single total or comma-separated currency totals (e.g. 965 USD, 765 EUR)</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>Two consolidated prompts: Financial Quality (date+currency+payment terms) and Entity Quality (country/region+supplier). Each returns structured 3-point insights per panel.</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>Fuzzy threshold: 0.75, max insight words: 10-15 per point</t>
+          <t>NA</t>
         </is>
       </c>
     </row>
@@ -2541,136 +2541,230 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
+          <t>Spend Bifurcation</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Expand the Spend Bifurcation panel (shown after Date panel)</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Session ID, table name</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Identifies spend column (reporting currency first, then local). Sums positive and negative spend separately. If local, groups by currency code.</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>JSON with type (reporting/local/none), positiveSpend, negativeSpend, or currencies array with per-currency pos/neg totals</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>If reporting: two-column table with Total Positive Spend and Total Negative Spend. If local: three-column table with Currency, Total +ve Spend, Total -ve Spend.</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>8. DQA</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Consolidated DQA (all panels)</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Automatic when user lands on the DQA step</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Session ID, API key, table name, optional date/country column overrides</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>First calls collect_column_samples + suggest_columns_ai to get AI column suggestions (outside lock). Then runs all seven DQA panels in parallel via run_dqa_all_sql, passing AI-suggested columns as defaults for currency, payment terms, and supplier panels. Each panel returns its available columns list for dropdown population.</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>JSON dict keyed by panel name with complete results including AI insights as 3-element arrays</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>All DQA panels render together. Currency, Payment Terms, and Supplier panels each show a dropdown pre-filled with the AI-suggested column. User can switch columns in any dropdown to trigger a single-panel rerun.</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Two consolidated prompts: Financial Quality (date+currency+payment terms) and Entity Quality (country/region+supplier). Each returns structured 3-point insights per panel.</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Fuzzy threshold: 0.75, max insight words: 10-15 per point</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>8. DQA</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
           <t>AI Column Suggestions</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr">
+      <c r="C43" t="inlineStr">
         <is>
           <t>None ? runs automatically when the user starts the assessment</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr">
+      <c r="D43" t="inlineStr">
         <is>
           <t>All column names from the working table plus 5 sample values per column, API key</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr">
+      <c r="E43" t="inlineStr">
         <is>
           <t>collect_column_samples reads column names and samples under session lock. suggest_columns_ai sends them to the LLM outside the lock and returns the top-3 most likely columns per role (date, currency, payment_terms, country, vendor_name).</t>
         </is>
       </c>
-      <c r="F41" t="inlineStr">
+      <c r="F43" t="inlineStr">
         <is>
           <t>JSON dict keyed by role, each value a list of up to 3 column names ordered by confidence</t>
         </is>
       </c>
-      <c r="G41" t="inlineStr">
+      <c r="G43" t="inlineStr">
         <is>
           <t>No direct UI; the suggested columns pre-fill the default selections and dropdown options for each analysis panel</t>
         </is>
       </c>
-      <c r="H41" t="inlineStr">
+      <c r="H43" t="inlineStr">
         <is>
           <t>System prompt lists every role with a description. User prompt contains each column name with 5 sample values. LLM returns JSON mapping each role to an ordered array of top-3 column names.</t>
         </is>
       </c>
-      <c r="I41" t="inlineStr">
+      <c r="I43" t="inlineStr">
         <is>
           <t>sample_size=5 rows per column; model from call_ai_json config</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="20" t="inlineStr">
+    <row r="44">
+      <c r="A44" s="20" t="inlineStr">
         <is>
           <t>Cross-cutting</t>
         </is>
       </c>
-      <c r="B42" s="21" t="inlineStr">
+      <c r="B44" s="21" t="inlineStr">
         <is>
           <t>Chat assistant</t>
         </is>
       </c>
-      <c r="C42" s="5" t="inlineStr">
+      <c r="C44" s="5" t="inlineStr">
         <is>
           <t>User opens chat panel and types a question at any step.</t>
         </is>
       </c>
-      <c r="D42" s="5" t="inlineStr">
+      <c r="D44" s="5" t="inlineStr">
         <is>
           <t>sessionId, message, context (auto-built from current stage, selected item, meta), apiKey, optional messages history.</t>
         </is>
       </c>
-      <c r="E42" s="5" t="inlineStr">
+      <c r="E44" s="5" t="inlineStr">
         <is>
           <t>System prompt defines the assistant as a procurement data expert embedded in DataStitcher. Context block injected with current stage data (counts, samples, groups, merge fields). Last 12 history messages included. Response is plain text (no JSON mode).</t>
         </is>
       </c>
-      <c r="F42" s="5" t="inlineStr">
+      <c r="F44" s="5" t="inlineStr">
         <is>
           <t>{content: "reply text"} via SSE (one message then [DONE]).</t>
         </is>
       </c>
-      <c r="G42" s="5" t="inlineStr">
+      <c r="G44" s="5" t="inlineStr">
         <is>
           <t>Chat panel with conversational AI assistant. Responds with procurement-aware advice, references actual column names and data from context.</t>
         </is>
       </c>
-      <c r="H42" s="5" t="inlineStr">
+      <c r="H44" s="5" t="inlineStr">
         <is>
           <t>System: "You are a concise data assistant embedded in DataStitcher, with deep expertise in procurement and supply chain data... Rules: be concise, 2-4 paragraphs max, plain language, reference actual column names... Procurement perspective: use procurement terminology (spend analysis, suppliers, categories, PO, invoices, contracts, OTIF, DPO, maverick spend, tail spend...)"
 User: The user's message.
 Context: Auto-built JSON with stage, meta, samples.</t>
         </is>
       </c>
-      <c r="I42" s="5" t="inlineStr">
+      <c r="I44" s="5" t="inlineStr">
         <is>
           <t>Last 12 history messages. AI cache TTL = 300s. AI retry attempts = 3.</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="20" t="inlineStr">
+    <row r="45">
+      <c r="A45" s="20" t="inlineStr">
         <is>
           <t>Cross-cutting</t>
         </is>
       </c>
-      <c r="B43" s="21" t="inlineStr">
+      <c r="B45" s="21" t="inlineStr">
         <is>
           <t>Group Insights (pipeline)</t>
         </is>
       </c>
-      <c r="C43" s="4" t="inlineStr">
+      <c r="C45" s="4" t="inlineStr">
         <is>
           <t>Currently not exposed in UI — backend-only pipeline.</t>
         </is>
       </c>
-      <c r="D43" s="4" t="inlineStr">
+      <c r="D45" s="4" t="inlineStr">
         <is>
           <t>sessionId, apiKey, groupIds.</t>
         </is>
       </c>
-      <c r="E43" s="4" t="inlineStr">
+      <c r="E45" s="4" t="inlineStr">
         <is>
           <t>Multi-step AI pipeline per group: (1) Data Profiler — column stats → data description, column roles, domain keywords. (2) Quality Auditor — scores quality 0–100, identifies issues by severity, recommends fixes. (3) Analytics Strategist — suggests up to 5 slices (GROUP BY dimension + aggregation). SQL executed for each slice (LIMIT 15 rows). (4) Insight Synthesizer — combines everything into top 3–5 findings with specific numbers. Cross-group: Cross-Group Synthesizer — narrative about how groups relate, merge hints.</t>
         </is>
       </c>
-      <c r="F43" s="4" t="inlineStr">
+      <c r="F45" s="4" t="inlineStr">
         <is>
           <t>Per-group: summary, topInsights, suggestedActions, qualityScore, issues. Cross-group: narrative, mergeHints.</t>
         </is>
       </c>
-      <c r="G43" s="4" t="inlineStr">
+      <c r="G45" s="4" t="inlineStr">
         <is>
           <t>Not rendered in current UI.</t>
         </is>
       </c>
-      <c r="H43" s="4" t="inlineStr">
+      <c r="H45" s="4" t="inlineStr">
         <is>
           <t>Profiler, Auditor, Strategist, Synthesizer, Cross-Group Synthesizer — each has a dedicated system prompt (see insight prompt chain). All return structured JSON.</t>
         </is>
       </c>
-      <c r="I43" s="4" t="inlineStr">
+      <c r="I45" s="4" t="inlineStr">
         <is>
           <t>Strategist slices capped at 5. Slice SQL LIMIT 15. Cross-group value overlap slice = 15. AI pool workers up to 6.</t>
         </is>

</xml_diff>